<commit_message>
BP 1999 und Pfad Fxes
</commit_message>
<xml_diff>
--- a/web/data/records_kriterien.xlsx
+++ b/web/data/records_kriterien.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\utilities\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14844F7B-1CCA-4917-B1F1-7A3F7DF9D036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB51B59-528E-4AEB-BE05-F671454C5529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" firstSheet="1" activeTab="3" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="687" activeTab="9" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
   <sheets>
     <sheet name="DR" sheetId="9" r:id="rId1"/>
@@ -1701,16 +1701,13 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1722,15 +1719,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1739,27 +1727,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1803,6 +1770,39 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
@@ -1930,6 +1930,58 @@
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1954,6 +2006,54 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1978,6 +2078,30 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2114,75 +2238,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -4232,79 +4287,60 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -4317,43 +4353,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4369,102 +4369,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="201" headerRowBorderDxfId="200" tableBorderDxfId="199">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="212" headerRowBorderDxfId="211" tableBorderDxfId="210">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="198">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="209">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="197"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="196"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="195"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="194"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="193"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="192"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="191"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="190"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="208"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="207"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="206"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="205"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="204"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="203"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="202"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="201"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="189"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="188"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="187"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="186"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="185"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="184"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="183"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="182"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="181"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="180"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="179"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="178"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="177"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="176"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="175"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="174"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="173"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="172"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="171"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="170"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="169"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="168"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="167"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="166"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="165"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="164"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="163"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="162"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="161"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="160"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="159"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="158"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="157"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="156"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="155"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="154"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="153"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="200"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="199"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="198"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="197"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="196"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="195"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="194"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="193"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="192"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="191"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="190"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="189"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="188"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="187"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="186"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="185"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="184"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="183"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="182"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="181"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="180"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="179"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="178"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="177"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="176"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="175"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="174"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="173"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="172"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="171"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="170"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="169"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="168"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="167"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="166"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="165"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="164"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="152" dataDxfId="150" headerRowBorderDxfId="151" tableBorderDxfId="149">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="163" dataDxfId="161" headerRowBorderDxfId="162" tableBorderDxfId="160">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="148"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="147"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="146"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="145"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="144"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="143"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="142"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="141"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="140"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="139"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="138"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="137"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="136"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="159"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="158"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="157"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="156"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="155"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="154"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="153"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="152"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="151"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="150"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="149"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="148"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="147"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="135" headerRowBorderDxfId="134" tableBorderDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="146" headerRowBorderDxfId="145" tableBorderDxfId="144">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="132">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="143">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="131"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="130"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="129"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="128"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="127"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="126"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="125"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="142"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="141"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="140"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="139"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="138"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="137"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="136"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="135"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -4475,7 +4475,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="235" dataDxfId="234">
   <autoFilter ref="A1:U3" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4500,64 +4500,64 @@
     <filterColumn colId="20" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="120"/>
-    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="119"/>
-    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="117"/>
-    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="116"/>
-    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="115"/>
-    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="114"/>
-    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="113"/>
-    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="112"/>
-    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="111"/>
-    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="110"/>
-    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="109"/>
-    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="108"/>
-    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="107"/>
-    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="106"/>
-    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="105"/>
-    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="104"/>
-    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="103"/>
-    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="102"/>
-    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="101"/>
+    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="233"/>
+    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="232"/>
+    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="231"/>
+    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="230"/>
+    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="229"/>
+    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="228"/>
+    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="227"/>
+    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="226"/>
+    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="225"/>
+    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="224"/>
+    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="223"/>
+    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="222"/>
+    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="221"/>
+    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="220"/>
+    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="219"/>
+    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="218"/>
+    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="217"/>
+    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="216"/>
+    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="215"/>
+    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="214"/>
+    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="213"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="134" dataDxfId="133">
   <autoFilter ref="A1:U7" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="91"/>
-    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="87"/>
-    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="86"/>
-    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="85"/>
-    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="84"/>
-    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="82"/>
-    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="81"/>
-    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="80"/>
-    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="79"/>
-    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="132"/>
+    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="131"/>
+    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="130"/>
+    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="129"/>
+    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="128"/>
+    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="127"/>
+    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="126"/>
+    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="125"/>
+    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="124"/>
+    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="123"/>
+    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="122"/>
+    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="121"/>
+    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="120"/>
+    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="119"/>
+    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="118"/>
+    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="117"/>
+    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="116"/>
+    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="115"/>
+    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="114"/>
+    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="113"/>
+    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="112"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
   <autoFilter ref="A1:X7" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4585,37 +4585,37 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="67"/>
-    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="66"/>
-    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="65"/>
-    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="64"/>
-    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="63"/>
-    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="62"/>
-    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="61"/>
-    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="60"/>
-    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="59"/>
-    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="58"/>
-    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="57"/>
-    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="56"/>
-    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="55"/>
-    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="54"/>
-    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="53"/>
-    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="105"/>
+    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="104"/>
+    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="103"/>
+    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="102"/>
+    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="101"/>
+    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="100"/>
+    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="99"/>
+    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="98"/>
+    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="97"/>
+    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="96"/>
+    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="95"/>
+    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="94"/>
+    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="93"/>
+    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="92"/>
+    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="91"/>
+    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="90"/>
+    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="89"/>
+    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="88"/>
+    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="87"/>
+    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
   <autoFilter ref="A1:X3" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4643,71 +4643,71 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="83"/>
+    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="74"/>
+    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="73"/>
+    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="72"/>
+    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="71"/>
+    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="70"/>
+    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="69"/>
+    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="68"/>
+    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="67"/>
+    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="66"/>
+    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="65"/>
+    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="64"/>
+    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="63"/>
+    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="62"/>
+    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="61"/>
+    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="235" dataDxfId="234">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
   <autoFilter ref="A1:AF37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
   <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="233"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="232"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="231"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="230"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="229"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="228"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="227"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="226"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="225"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="224"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="223"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="222"/>
-    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="221"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="220"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="219"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="218"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="217"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="216"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="215"/>
-    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="214"/>
-    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="213"/>
-    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="212"/>
-    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="211"/>
-    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="210"/>
-    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="209"/>
-    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="208"/>
-    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="207"/>
-    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="206"/>
-    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="205"/>
-    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="204"/>
-    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="203"/>
-    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="202"/>
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="49"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="46"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="45"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="44"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="43"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="42"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="41"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="40"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="39"/>
+    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="38"/>
+    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="37"/>
+    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="36"/>
+    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="35"/>
+    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="34"/>
+    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="33"/>
+    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="32"/>
+    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="31"/>
+    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="30"/>
+    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="29"/>
+    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="28"/>
+    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="27"/>
+    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5049,9 +5049,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0519F5DB-31A0-4819-8E86-33B1F16466A6}">
   <sheetPr codeName="Tabelle6"/>
   <dimension ref="A1:AW31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.265625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
@@ -5120,7 +5120,7 @@
       <c r="AV1" s="10"/>
       <c r="AW1" s="10"/>
     </row>
-    <row r="2" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -5187,7 +5187,7 @@
       <c r="AV2" s="11"/>
       <c r="AW2" s="11"/>
     </row>
-    <row r="3" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>67</v>
       </c>
@@ -5248,7 +5248,7 @@
       <c r="AV3" s="11"/>
       <c r="AW3" s="11"/>
     </row>
-    <row r="4" spans="1:49" s="19" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:49" s="19" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
@@ -5397,7 +5397,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2000</v>
       </c>
@@ -5450,7 +5450,7 @@
       <c r="AV5" s="3"/>
       <c r="AW5" s="3"/>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f t="shared" ref="A6:A31" si="0">A5+1</f>
         <v>2001</v>
@@ -5528,7 +5528,7 @@
       <c r="AV6" s="4"/>
       <c r="AW6" s="4"/>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>2002</v>
@@ -5606,7 +5606,7 @@
       <c r="AV7" s="3"/>
       <c r="AW7" s="3"/>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>2003</v>
@@ -5684,7 +5684,7 @@
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>2004</v>
@@ -5762,7 +5762,7 @@
       <c r="AV9" s="3"/>
       <c r="AW9" s="3"/>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>2005</v>
@@ -5840,7 +5840,7 @@
       <c r="AV10" s="4"/>
       <c r="AW10" s="4"/>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>2006</v>
@@ -5918,7 +5918,7 @@
       <c r="AV11" s="3"/>
       <c r="AW11" s="3"/>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>2007</v>
@@ -6040,7 +6040,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>2008</v>
@@ -6162,7 +6162,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>2009</v>
@@ -6284,7 +6284,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>2010</v>
@@ -6406,7 +6406,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>2011</v>
@@ -6540,7 +6540,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <f t="shared" si="0"/>
         <v>2012</v>
@@ -6674,7 +6674,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
         <v>2013</v>
@@ -6808,7 +6808,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <f t="shared" si="0"/>
         <v>2014</v>
@@ -6942,7 +6942,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <f t="shared" si="0"/>
         <v>2015</v>
@@ -7076,7 +7076,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <f t="shared" si="0"/>
         <v>2016</v>
@@ -7210,7 +7210,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <f t="shared" si="0"/>
         <v>2017</v>
@@ -7344,7 +7344,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <f t="shared" si="0"/>
         <v>2018</v>
@@ -7478,7 +7478,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <f t="shared" si="0"/>
         <v>2019</v>
@@ -7612,7 +7612,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <f t="shared" si="0"/>
         <v>2020</v>
@@ -7762,7 +7762,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <f t="shared" si="0"/>
         <v>2021</v>
@@ -7912,7 +7912,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <f t="shared" si="0"/>
         <v>2022</v>
@@ -8062,7 +8062,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -8212,7 +8212,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -8362,7 +8362,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -8512,7 +8512,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -8728,18 +8728,18 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="84.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="84.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>191</v>
       </c>
@@ -8765,7 +8765,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="36">
         <v>46124</v>
       </c>
@@ -8788,7 +8788,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="36">
         <v>46124</v>
       </c>
@@ -8811,7 +8811,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="36">
         <v>46186</v>
       </c>
@@ -8834,7 +8834,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="36">
         <v>46187</v>
       </c>
@@ -8857,7 +8857,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="36">
         <v>46199</v>
       </c>
@@ -8883,7 +8883,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="36">
         <v>46201</v>
       </c>
@@ -8906,7 +8906,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="36">
         <v>46228</v>
       </c>
@@ -8946,17 +8946,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB2B168-68B3-410F-B4A6-8D511F9C32E0}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.265625" customWidth="1"/>
-    <col min="2" max="5" width="18.73046875" customWidth="1"/>
-    <col min="6" max="6" width="21.1328125" customWidth="1"/>
-    <col min="7" max="11" width="18.73046875" customWidth="1"/>
-    <col min="12" max="12" width="22.1328125" customWidth="1"/>
-    <col min="13" max="13" width="18.73046875" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="11" width="18.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.140625" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -9038,7 +9038,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>15</v>
       </c>
@@ -9079,7 +9079,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -9120,7 +9120,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2000</v>
       </c>
@@ -9137,7 +9137,7 @@
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f t="shared" ref="A6:A32" si="0">A5+1</f>
         <v>2001</v>
@@ -9155,7 +9155,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>2002</v>
@@ -9173,7 +9173,7 @@
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>2003</v>
@@ -9191,7 +9191,7 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>2004</v>
@@ -9209,7 +9209,7 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>2005</v>
@@ -9227,7 +9227,7 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>2006</v>
@@ -9245,7 +9245,7 @@
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>2007</v>
@@ -9263,7 +9263,7 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>2008</v>
@@ -9281,7 +9281,7 @@
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>2009</v>
@@ -9299,7 +9299,7 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>2010</v>
@@ -9317,7 +9317,7 @@
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>2011</v>
@@ -9335,7 +9335,7 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <f t="shared" si="0"/>
         <v>2012</v>
@@ -9353,7 +9353,7 @@
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
         <v>2013</v>
@@ -9371,7 +9371,7 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <f t="shared" si="0"/>
         <v>2014</v>
@@ -9389,7 +9389,7 @@
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <f t="shared" si="0"/>
         <v>2015</v>
@@ -9431,7 +9431,7 @@
         <v>1.3592592592592591E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <f t="shared" si="0"/>
         <v>2016</v>
@@ -9473,7 +9473,7 @@
         <v>1.3592592592592591E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <f t="shared" si="0"/>
         <v>2017</v>
@@ -9515,7 +9515,7 @@
         <v>1.3577546296296298E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <f t="shared" si="0"/>
         <v>2018</v>
@@ -9557,7 +9557,7 @@
         <v>1.3577546296296298E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <f t="shared" si="0"/>
         <v>2019</v>
@@ -9599,7 +9599,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <f t="shared" si="0"/>
         <v>2020</v>
@@ -9641,7 +9641,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <f t="shared" si="0"/>
         <v>2021</v>
@@ -9683,7 +9683,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <f t="shared" si="0"/>
         <v>2022</v>
@@ -9725,7 +9725,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -9767,7 +9767,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -9809,7 +9809,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -9851,7 +9851,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -9893,7 +9893,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -9968,17 +9968,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC5FFB6C-7DEA-4C95-82B5-1769BD3934D8}">
   <sheetPr codeName="Tabelle2"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.86328125" customWidth="1"/>
-    <col min="2" max="5" width="18.73046875" customWidth="1"/>
-    <col min="6" max="6" width="21.1328125" customWidth="1"/>
-    <col min="7" max="11" width="18.73046875" customWidth="1"/>
-    <col min="12" max="12" width="22.1328125" customWidth="1"/>
-    <col min="13" max="13" width="18.73046875" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="2" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="11" width="18.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.140625" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
@@ -10019,7 +10019,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -10060,7 +10060,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>15</v>
       </c>
@@ -10101,7 +10101,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -10142,7 +10142,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2000</v>
       </c>
@@ -10159,7 +10159,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f t="shared" ref="A6:A31" si="0">A5+1</f>
         <v>2001</v>
@@ -10189,7 +10189,7 @@
         <v>1.3629629629629632E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>2002</v>
@@ -10231,7 +10231,7 @@
         <v>1.3629629629629632E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>2003</v>
@@ -10273,7 +10273,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>2004</v>
@@ -10315,7 +10315,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>2005</v>
@@ -10357,7 +10357,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>2006</v>
@@ -10399,7 +10399,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>2007</v>
@@ -10441,7 +10441,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>2008</v>
@@ -10483,7 +10483,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>2009</v>
@@ -10525,7 +10525,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>2010</v>
@@ -10567,7 +10567,7 @@
         <v>1.3306712962962966E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>2011</v>
@@ -10609,7 +10609,7 @@
         <v>1.3306712962962966E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <f t="shared" si="0"/>
         <v>2012</v>
@@ -10651,7 +10651,7 @@
         <v>1.3306712962962966E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
         <v>2013</v>
@@ -10693,7 +10693,7 @@
         <v>1.312962962962963E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <f t="shared" si="0"/>
         <v>2014</v>
@@ -10735,7 +10735,7 @@
         <v>1.312962962962963E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <f t="shared" si="0"/>
         <v>2015</v>
@@ -10777,7 +10777,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <f t="shared" si="0"/>
         <v>2016</v>
@@ -10819,7 +10819,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <f t="shared" si="0"/>
         <v>2017</v>
@@ -10861,7 +10861,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <f t="shared" si="0"/>
         <v>2018</v>
@@ -10903,7 +10903,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <f t="shared" si="0"/>
         <v>2019</v>
@@ -10945,7 +10945,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <f t="shared" si="0"/>
         <v>2020</v>
@@ -10987,7 +10987,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <f t="shared" si="0"/>
         <v>2021</v>
@@ -11029,7 +11029,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <f t="shared" si="0"/>
         <v>2022</v>
@@ -11071,7 +11071,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -11113,7 +11113,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -11155,7 +11155,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -11197,7 +11197,7 @@
         <v>1.2931712962962962E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -11239,7 +11239,7 @@
         <v>1.2931712962962962E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <f>A31+1</f>
         <v>2027</v>
@@ -11316,30 +11316,30 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:U3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.73046875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.73046875" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" customWidth="1"/>
     <col min="15" max="16" width="19" customWidth="1"/>
-    <col min="17" max="17" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="22.265625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.73046875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="47.265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="47.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>127</v>
       </c>
@@ -11404,7 +11404,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>163</v>
       </c>
@@ -11461,7 +11461,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>164</v>
       </c>
@@ -11532,30 +11532,30 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:U7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.73046875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.73046875" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" customWidth="1"/>
     <col min="15" max="16" width="19" customWidth="1"/>
-    <col min="17" max="17" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="22.265625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.73046875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="47.265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="47.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>127</v>
       </c>
@@ -11620,7 +11620,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>155</v>
       </c>
@@ -11681,7 +11681,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>156</v>
       </c>
@@ -11742,7 +11742,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>157</v>
       </c>
@@ -11803,7 +11803,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>158</v>
       </c>
@@ -11862,7 +11862,7 @@
       </c>
       <c r="U5" s="25"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>159</v>
       </c>
@@ -11921,7 +11921,7 @@
       </c>
       <c r="U6" s="25"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>160</v>
       </c>
@@ -11994,35 +11994,35 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:X7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.1328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.1328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12096,7 +12096,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>178</v>
       </c>
@@ -12166,7 +12166,7 @@
         <v>1.9623842592592592E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>179</v>
       </c>
@@ -12236,7 +12236,7 @@
         <v>1.8121527777777778E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>180</v>
       </c>
@@ -12306,7 +12306,7 @@
         <v>1.9979166666666665E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>181</v>
       </c>
@@ -12376,7 +12376,7 @@
         <v>1.7653935185185186E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>155</v>
       </c>
@@ -12446,7 +12446,7 @@
         <v>1.8998842592592594E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>156</v>
       </c>
@@ -12530,35 +12530,35 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:X3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="27" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="22" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="19.265625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12632,7 +12632,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>189</v>
       </c>
@@ -12702,7 +12702,7 @@
         <v>1.8332175925925925E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>190</v>
       </c>
@@ -12786,30 +12786,30 @@
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AF37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.86328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.19921875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.1328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12907,7 +12907,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>241</v>
       </c>
@@ -12981,7 +12981,7 @@
       <c r="AE2" s="106"/>
       <c r="AF2" s="106"/>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>241</v>
       </c>
@@ -13055,7 +13055,7 @@
       <c r="AE3" s="106"/>
       <c r="AF3" s="106"/>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>241</v>
       </c>
@@ -13129,7 +13129,7 @@
       <c r="AE4" s="106"/>
       <c r="AF4" s="106"/>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>233</v>
       </c>
@@ -13203,7 +13203,7 @@
       <c r="AE5" s="106"/>
       <c r="AF5" s="106"/>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>233</v>
       </c>
@@ -13277,7 +13277,7 @@
       <c r="AE6" s="106"/>
       <c r="AF6" s="106"/>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>233</v>
       </c>
@@ -13351,7 +13351,7 @@
       <c r="AE7" s="106"/>
       <c r="AF7" s="106"/>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
         <v>240</v>
       </c>
@@ -13425,7 +13425,7 @@
       <c r="AE8" s="106"/>
       <c r="AF8" s="106"/>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
         <v>240</v>
       </c>
@@ -13499,7 +13499,7 @@
       <c r="AE9" s="106"/>
       <c r="AF9" s="106"/>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
         <v>240</v>
       </c>
@@ -13573,7 +13573,7 @@
       <c r="AE10" s="106"/>
       <c r="AF10" s="106"/>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
         <v>239</v>
       </c>
@@ -13647,7 +13647,7 @@
       <c r="AE11" s="106"/>
       <c r="AF11" s="106"/>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
         <v>239</v>
       </c>
@@ -13721,7 +13721,7 @@
       <c r="AE12" s="106"/>
       <c r="AF12" s="106"/>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
         <v>239</v>
       </c>
@@ -13795,7 +13795,7 @@
       <c r="AE13" s="106"/>
       <c r="AF13" s="106"/>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
         <v>222</v>
       </c>
@@ -13881,7 +13881,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
         <v>222</v>
       </c>
@@ -13969,7 +13969,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
         <v>222</v>
       </c>
@@ -14057,7 +14057,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
         <v>220</v>
       </c>
@@ -14143,7 +14143,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
         <v>220</v>
       </c>
@@ -14231,7 +14231,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>220</v>
       </c>
@@ -14319,7 +14319,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
         <v>243</v>
       </c>
@@ -14405,7 +14405,7 @@
       <c r="AE20" s="106"/>
       <c r="AF20" s="106"/>
     </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
         <v>243</v>
       </c>
@@ -14491,7 +14491,7 @@
       <c r="AE21" s="106"/>
       <c r="AF21" s="106"/>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
         <v>243</v>
       </c>
@@ -14581,7 +14581,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
         <v>243</v>
       </c>
@@ -14671,7 +14671,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
         <v>243</v>
       </c>
@@ -14759,7 +14759,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
         <v>244</v>
       </c>
@@ -14845,7 +14845,7 @@
       <c r="AE25" s="106"/>
       <c r="AF25" s="106"/>
     </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>244</v>
       </c>
@@ -14931,7 +14931,7 @@
       <c r="AE26" s="106"/>
       <c r="AF26" s="106"/>
     </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
         <v>244</v>
       </c>
@@ -15021,7 +15021,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
         <v>244</v>
       </c>
@@ -15111,7 +15111,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
         <v>244</v>
       </c>
@@ -15199,7 +15199,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
         <v>245</v>
       </c>
@@ -15285,7 +15285,7 @@
       <c r="AE30" s="106"/>
       <c r="AF30" s="106"/>
     </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
         <v>245</v>
       </c>
@@ -15371,7 +15371,7 @@
       <c r="AE31" s="106"/>
       <c r="AF31" s="106"/>
     </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="25" t="s">
         <v>245</v>
       </c>
@@ -15457,7 +15457,7 @@
       <c r="AE32" s="106"/>
       <c r="AF32" s="106"/>
     </row>
-    <row r="33" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
         <v>245</v>
       </c>
@@ -15543,7 +15543,7 @@
       <c r="AE33" s="106"/>
       <c r="AF33" s="106"/>
     </row>
-    <row r="34" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
         <v>246</v>
       </c>
@@ -15629,7 +15629,7 @@
       <c r="AE34" s="106"/>
       <c r="AF34" s="106"/>
     </row>
-    <row r="35" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A35" s="25" t="s">
         <v>246</v>
       </c>
@@ -15715,7 +15715,7 @@
       <c r="AE35" s="106"/>
       <c r="AF35" s="106"/>
     </row>
-    <row r="36" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A36" s="25" t="s">
         <v>246</v>
       </c>
@@ -15801,7 +15801,7 @@
       <c r="AE36" s="106"/>
       <c r="AF36" s="106"/>
     </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A37" s="25" t="s">
         <v>246</v>
       </c>
@@ -15900,145 +15900,145 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A13DA696-49DD-4BFA-98FE-5C7770404E50}">
   <sheetPr codeName="Tabelle12"/>
   <dimension ref="A1:BZ45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.265625" customWidth="1"/>
-    <col min="2" max="2" width="32.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="26" width="9.59765625" customWidth="1"/>
-    <col min="28" max="28" width="32.3984375" bestFit="1" customWidth="1"/>
-    <col min="29" max="52" width="4.59765625" customWidth="1"/>
-    <col min="54" max="54" width="32.3984375" bestFit="1" customWidth="1"/>
-    <col min="55" max="78" width="9.59765625" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="26" width="9.5703125" customWidth="1"/>
+    <col min="28" max="28" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="52" width="4.5703125" customWidth="1"/>
+    <col min="54" max="54" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="55" max="78" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="126">
+    <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="107">
         <v>2025</v>
       </c>
       <c r="B1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="108" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="111" t="s">
+      <c r="D1" s="108"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="117" t="s">
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="113" t="s">
         <v>225</v>
       </c>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="109" t="s">
+      <c r="L1" s="114"/>
+      <c r="M1" s="114"/>
+      <c r="N1" s="115"/>
+      <c r="O1" s="133" t="s">
         <v>222</v>
       </c>
-      <c r="P1" s="109"/>
-      <c r="Q1" s="110"/>
-      <c r="R1" s="123" t="s">
+      <c r="P1" s="133"/>
+      <c r="Q1" s="134"/>
+      <c r="R1" s="135" t="s">
         <v>223</v>
       </c>
-      <c r="S1" s="124"/>
-      <c r="T1" s="124"/>
-      <c r="U1" s="124"/>
-      <c r="V1" s="125"/>
-      <c r="W1" s="120" t="s">
+      <c r="S1" s="136"/>
+      <c r="T1" s="136"/>
+      <c r="U1" s="136"/>
+      <c r="V1" s="137"/>
+      <c r="W1" s="138" t="s">
         <v>226</v>
       </c>
-      <c r="X1" s="121"/>
-      <c r="Y1" s="121"/>
-      <c r="Z1" s="122"/>
+      <c r="X1" s="139"/>
+      <c r="Y1" s="139"/>
+      <c r="Z1" s="140"/>
       <c r="AA1"/>
       <c r="AB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="127" t="s">
+      <c r="AC1" s="116" t="s">
         <v>227</v>
       </c>
-      <c r="AD1" s="127"/>
-      <c r="AE1" s="128"/>
-      <c r="AF1" s="129" t="s">
+      <c r="AD1" s="116"/>
+      <c r="AE1" s="117"/>
+      <c r="AF1" s="118" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="130"/>
-      <c r="AH1" s="130"/>
-      <c r="AI1" s="130"/>
-      <c r="AJ1" s="131"/>
-      <c r="AK1" s="132" t="s">
+      <c r="AG1" s="119"/>
+      <c r="AH1" s="119"/>
+      <c r="AI1" s="119"/>
+      <c r="AJ1" s="120"/>
+      <c r="AK1" s="121" t="s">
         <v>229</v>
       </c>
-      <c r="AL1" s="133"/>
-      <c r="AM1" s="133"/>
-      <c r="AN1" s="134"/>
-      <c r="AO1" s="135" t="s">
+      <c r="AL1" s="122"/>
+      <c r="AM1" s="122"/>
+      <c r="AN1" s="123"/>
+      <c r="AO1" s="124" t="s">
         <v>230</v>
       </c>
-      <c r="AP1" s="136"/>
-      <c r="AQ1" s="137"/>
-      <c r="AR1" s="138" t="s">
+      <c r="AP1" s="125"/>
+      <c r="AQ1" s="126"/>
+      <c r="AR1" s="127" t="s">
         <v>231</v>
       </c>
-      <c r="AS1" s="139"/>
-      <c r="AT1" s="139"/>
-      <c r="AU1" s="139"/>
-      <c r="AV1" s="140"/>
-      <c r="AW1" s="114" t="s">
+      <c r="AS1" s="128"/>
+      <c r="AT1" s="128"/>
+      <c r="AU1" s="128"/>
+      <c r="AV1" s="129"/>
+      <c r="AW1" s="130" t="s">
         <v>232</v>
       </c>
-      <c r="AX1" s="115"/>
-      <c r="AY1" s="115"/>
-      <c r="AZ1" s="116"/>
+      <c r="AX1" s="131"/>
+      <c r="AY1" s="131"/>
+      <c r="AZ1" s="132"/>
       <c r="BB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="107" t="s">
+      <c r="BC1" s="108" t="s">
         <v>233</v>
       </c>
-      <c r="BD1" s="107"/>
-      <c r="BE1" s="108"/>
-      <c r="BF1" s="111" t="s">
+      <c r="BD1" s="108"/>
+      <c r="BE1" s="109"/>
+      <c r="BF1" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="BG1" s="112"/>
-      <c r="BH1" s="112"/>
-      <c r="BI1" s="112"/>
-      <c r="BJ1" s="113"/>
-      <c r="BK1" s="117" t="s">
+      <c r="BG1" s="111"/>
+      <c r="BH1" s="111"/>
+      <c r="BI1" s="111"/>
+      <c r="BJ1" s="112"/>
+      <c r="BK1" s="113" t="s">
         <v>235</v>
       </c>
-      <c r="BL1" s="118"/>
-      <c r="BM1" s="118"/>
-      <c r="BN1" s="119"/>
-      <c r="BO1" s="109" t="s">
+      <c r="BL1" s="114"/>
+      <c r="BM1" s="114"/>
+      <c r="BN1" s="115"/>
+      <c r="BO1" s="133" t="s">
         <v>241</v>
       </c>
-      <c r="BP1" s="109"/>
-      <c r="BQ1" s="110"/>
-      <c r="BR1" s="123" t="s">
+      <c r="BP1" s="133"/>
+      <c r="BQ1" s="134"/>
+      <c r="BR1" s="135" t="s">
         <v>242</v>
       </c>
-      <c r="BS1" s="124"/>
-      <c r="BT1" s="124"/>
-      <c r="BU1" s="124"/>
-      <c r="BV1" s="125"/>
-      <c r="BW1" s="120" t="s">
+      <c r="BS1" s="136"/>
+      <c r="BT1" s="136"/>
+      <c r="BU1" s="136"/>
+      <c r="BV1" s="137"/>
+      <c r="BW1" s="138" t="s">
         <v>236</v>
       </c>
-      <c r="BX1" s="121"/>
-      <c r="BY1" s="121"/>
-      <c r="BZ1" s="122"/>
+      <c r="BX1" s="139"/>
+      <c r="BY1" s="139"/>
+      <c r="BZ1" s="140"/>
     </row>
-    <row r="2" spans="1:78" s="94" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="126"/>
+    <row r="2" spans="1:78" s="94" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="107"/>
       <c r="B2" s="46" t="s">
         <v>224</v>
       </c>
@@ -16338,8 +16338,8 @@
         <v>2001-1985</v>
       </c>
     </row>
-    <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="126"/>
+    <row r="3" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="107"/>
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
@@ -16591,8 +16591,8 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="126"/>
+    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A4" s="107"/>
       <c r="B4" s="47" t="s">
         <v>185</v>
       </c>
@@ -16843,8 +16843,8 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="126"/>
+    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A5" s="107"/>
       <c r="B5" s="47" t="s">
         <v>186</v>
       </c>
@@ -17095,8 +17095,8 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="126"/>
+    <row r="6" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A6" s="107"/>
       <c r="B6" s="47" t="s">
         <v>187</v>
       </c>
@@ -17347,8 +17347,8 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="126"/>
+    <row r="7" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A7" s="107"/>
       <c r="B7" s="47" t="s">
         <v>188</v>
       </c>
@@ -17599,8 +17599,8 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="126"/>
+    <row r="8" spans="1:78" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="107"/>
       <c r="B8" s="50" t="s">
         <v>4</v>
       </c>
@@ -17851,134 +17851,134 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
-    <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="126">
+    <row r="9" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:78" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="107">
         <v>2026</v>
       </c>
       <c r="B10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="107" t="s">
+      <c r="C10" s="108" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="107"/>
-      <c r="E10" s="108"/>
-      <c r="F10" s="111" t="s">
+      <c r="D10" s="108"/>
+      <c r="E10" s="109"/>
+      <c r="F10" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="112"/>
-      <c r="H10" s="112"/>
-      <c r="I10" s="112"/>
-      <c r="J10" s="113"/>
-      <c r="K10" s="117" t="s">
+      <c r="G10" s="111"/>
+      <c r="H10" s="111"/>
+      <c r="I10" s="111"/>
+      <c r="J10" s="112"/>
+      <c r="K10" s="113" t="s">
         <v>225</v>
       </c>
-      <c r="L10" s="118"/>
-      <c r="M10" s="118"/>
-      <c r="N10" s="119"/>
-      <c r="O10" s="109" t="s">
+      <c r="L10" s="114"/>
+      <c r="M10" s="114"/>
+      <c r="N10" s="115"/>
+      <c r="O10" s="133" t="s">
         <v>222</v>
       </c>
-      <c r="P10" s="109"/>
-      <c r="Q10" s="110"/>
-      <c r="R10" s="123" t="s">
+      <c r="P10" s="133"/>
+      <c r="Q10" s="134"/>
+      <c r="R10" s="135" t="s">
         <v>223</v>
       </c>
-      <c r="S10" s="124"/>
-      <c r="T10" s="124"/>
-      <c r="U10" s="124"/>
-      <c r="V10" s="125"/>
-      <c r="W10" s="120" t="s">
+      <c r="S10" s="136"/>
+      <c r="T10" s="136"/>
+      <c r="U10" s="136"/>
+      <c r="V10" s="137"/>
+      <c r="W10" s="138" t="s">
         <v>226</v>
       </c>
-      <c r="X10" s="121"/>
-      <c r="Y10" s="121"/>
-      <c r="Z10" s="122"/>
+      <c r="X10" s="139"/>
+      <c r="Y10" s="139"/>
+      <c r="Z10" s="140"/>
       <c r="AB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="127" t="s">
+      <c r="AC10" s="116" t="s">
         <v>227</v>
       </c>
-      <c r="AD10" s="127"/>
-      <c r="AE10" s="128"/>
-      <c r="AF10" s="129" t="s">
+      <c r="AD10" s="116"/>
+      <c r="AE10" s="117"/>
+      <c r="AF10" s="118" t="s">
         <v>228</v>
       </c>
-      <c r="AG10" s="130"/>
-      <c r="AH10" s="130"/>
-      <c r="AI10" s="130"/>
-      <c r="AJ10" s="131"/>
-      <c r="AK10" s="132" t="s">
+      <c r="AG10" s="119"/>
+      <c r="AH10" s="119"/>
+      <c r="AI10" s="119"/>
+      <c r="AJ10" s="120"/>
+      <c r="AK10" s="121" t="s">
         <v>229</v>
       </c>
-      <c r="AL10" s="133"/>
-      <c r="AM10" s="133"/>
-      <c r="AN10" s="134"/>
-      <c r="AO10" s="135" t="s">
+      <c r="AL10" s="122"/>
+      <c r="AM10" s="122"/>
+      <c r="AN10" s="123"/>
+      <c r="AO10" s="124" t="s">
         <v>230</v>
       </c>
-      <c r="AP10" s="136"/>
-      <c r="AQ10" s="137"/>
-      <c r="AR10" s="138" t="s">
+      <c r="AP10" s="125"/>
+      <c r="AQ10" s="126"/>
+      <c r="AR10" s="127" t="s">
         <v>231</v>
       </c>
-      <c r="AS10" s="139"/>
-      <c r="AT10" s="139"/>
-      <c r="AU10" s="139"/>
-      <c r="AV10" s="140"/>
-      <c r="AW10" s="114" t="s">
+      <c r="AS10" s="128"/>
+      <c r="AT10" s="128"/>
+      <c r="AU10" s="128"/>
+      <c r="AV10" s="129"/>
+      <c r="AW10" s="130" t="s">
         <v>232</v>
       </c>
-      <c r="AX10" s="115"/>
-      <c r="AY10" s="115"/>
-      <c r="AZ10" s="116"/>
+      <c r="AX10" s="131"/>
+      <c r="AY10" s="131"/>
+      <c r="AZ10" s="132"/>
       <c r="BB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="107" t="s">
+      <c r="BC10" s="108" t="s">
         <v>233</v>
       </c>
-      <c r="BD10" s="107"/>
-      <c r="BE10" s="108"/>
-      <c r="BF10" s="111" t="s">
+      <c r="BD10" s="108"/>
+      <c r="BE10" s="109"/>
+      <c r="BF10" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="BG10" s="112"/>
-      <c r="BH10" s="112"/>
-      <c r="BI10" s="112"/>
-      <c r="BJ10" s="113"/>
-      <c r="BK10" s="117" t="s">
+      <c r="BG10" s="111"/>
+      <c r="BH10" s="111"/>
+      <c r="BI10" s="111"/>
+      <c r="BJ10" s="112"/>
+      <c r="BK10" s="113" t="s">
         <v>235</v>
       </c>
-      <c r="BL10" s="118"/>
-      <c r="BM10" s="118"/>
-      <c r="BN10" s="119"/>
-      <c r="BO10" s="109" t="s">
+      <c r="BL10" s="114"/>
+      <c r="BM10" s="114"/>
+      <c r="BN10" s="115"/>
+      <c r="BO10" s="133" t="s">
         <v>241</v>
       </c>
-      <c r="BP10" s="109"/>
-      <c r="BQ10" s="110"/>
-      <c r="BR10" s="123" t="s">
+      <c r="BP10" s="133"/>
+      <c r="BQ10" s="134"/>
+      <c r="BR10" s="135" t="s">
         <v>242</v>
       </c>
-      <c r="BS10" s="124"/>
-      <c r="BT10" s="124"/>
-      <c r="BU10" s="124"/>
-      <c r="BV10" s="125"/>
-      <c r="BW10" s="120" t="s">
+      <c r="BS10" s="136"/>
+      <c r="BT10" s="136"/>
+      <c r="BU10" s="136"/>
+      <c r="BV10" s="137"/>
+      <c r="BW10" s="138" t="s">
         <v>236</v>
       </c>
-      <c r="BX10" s="121"/>
-      <c r="BY10" s="121"/>
-      <c r="BZ10" s="122"/>
+      <c r="BX10" s="139"/>
+      <c r="BY10" s="139"/>
+      <c r="BZ10" s="140"/>
     </row>
-    <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="126"/>
+    <row r="11" spans="1:78" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="107"/>
       <c r="B11" s="46" t="s">
         <v>224</v>
       </c>
@@ -18278,8 +18278,8 @@
         <v>2001-1985</v>
       </c>
     </row>
-    <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="126"/>
+    <row r="12" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="107"/>
       <c r="B12" s="47" t="s">
         <v>0</v>
       </c>
@@ -18530,8 +18530,8 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="126"/>
+    <row r="13" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A13" s="107"/>
       <c r="B13" s="47" t="s">
         <v>185</v>
       </c>
@@ -18782,8 +18782,8 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="126"/>
+    <row r="14" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A14" s="107"/>
       <c r="B14" s="47" t="s">
         <v>186</v>
       </c>
@@ -19034,8 +19034,8 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="126"/>
+    <row r="15" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="A15" s="107"/>
       <c r="B15" s="47" t="s">
         <v>187</v>
       </c>
@@ -19286,8 +19286,8 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="126"/>
+    <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="107"/>
       <c r="B16" s="47" t="s">
         <v>188</v>
       </c>
@@ -19538,8 +19538,8 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="126"/>
+    <row r="17" spans="1:78" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="107"/>
       <c r="B17" s="50" t="s">
         <v>4</v>
       </c>
@@ -19790,7 +19790,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C18" s="30"/>
       <c r="O18" s="30"/>
       <c r="T18" s="33"/>
@@ -19799,7 +19799,7 @@
       <c r="X18" s="30"/>
       <c r="AD18" s="30"/>
     </row>
-    <row r="21" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C21" s="29"/>
       <c r="D21" s="32"/>
       <c r="E21" s="32"/>
@@ -19819,7 +19819,7 @@
       <c r="AF21" s="35"/>
       <c r="AG21" s="35"/>
     </row>
-    <row r="22" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C22" s="30"/>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -19839,7 +19839,7 @@
       <c r="AF22" s="31"/>
       <c r="AG22" s="31"/>
     </row>
-    <row r="23" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C23" s="30"/>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -19859,7 +19859,7 @@
       <c r="AF23" s="31"/>
       <c r="AG23" s="31"/>
     </row>
-    <row r="24" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C24" s="30"/>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -19879,7 +19879,7 @@
       <c r="AF24" s="31"/>
       <c r="AG24" s="31"/>
     </row>
-    <row r="25" spans="1:78" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:78" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="30"/>
       <c r="D25" s="31"/>
       <c r="E25" s="31"/>
@@ -19899,7 +19899,7 @@
       <c r="AF25" s="31"/>
       <c r="AG25" s="31"/>
     </row>
-    <row r="26" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C26" s="30"/>
       <c r="D26" s="31"/>
       <c r="E26" s="31"/>
@@ -19919,7 +19919,7 @@
       <c r="AF26" s="31"/>
       <c r="AG26" s="31"/>
     </row>
-    <row r="27" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C27" s="30"/>
       <c r="D27" s="31"/>
       <c r="E27" s="31"/>
@@ -19939,7 +19939,7 @@
       <c r="AF27" s="31"/>
       <c r="AG27" s="31"/>
     </row>
-    <row r="30" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C30" s="29"/>
       <c r="D30" s="32"/>
       <c r="E30" s="32"/>
@@ -19948,7 +19948,7 @@
       <c r="H30" s="32"/>
       <c r="P30" s="33"/>
     </row>
-    <row r="31" spans="1:78" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:78" x14ac:dyDescent="0.25">
       <c r="C31" s="30"/>
       <c r="D31" s="31"/>
       <c r="E31" s="31"/>
@@ -19956,7 +19956,7 @@
       <c r="G31" s="31"/>
       <c r="H31" s="31"/>
     </row>
-    <row r="40" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="40" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C40" s="30"/>
       <c r="D40" s="31"/>
       <c r="E40" s="31"/>
@@ -19964,7 +19964,7 @@
       <c r="G40" s="31"/>
       <c r="H40" s="31"/>
     </row>
-    <row r="41" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="41" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C41" s="30"/>
       <c r="D41" s="31"/>
       <c r="E41" s="31"/>
@@ -19972,7 +19972,7 @@
       <c r="G41" s="31"/>
       <c r="H41" s="31"/>
     </row>
-    <row r="42" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="42" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C42" s="30"/>
       <c r="D42" s="31"/>
       <c r="E42" s="31"/>
@@ -19980,7 +19980,7 @@
       <c r="G42" s="31"/>
       <c r="H42" s="31"/>
     </row>
-    <row r="43" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="43" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C43" s="30"/>
       <c r="D43" s="31"/>
       <c r="E43" s="31"/>
@@ -19988,7 +19988,7 @@
       <c r="G43" s="31"/>
       <c r="H43" s="31"/>
     </row>
-    <row r="44" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="44" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C44" s="30"/>
       <c r="D44" s="31"/>
       <c r="E44" s="31"/>
@@ -19996,7 +19996,7 @@
       <c r="G44" s="31"/>
       <c r="H44" s="31"/>
     </row>
-    <row r="45" spans="3:8" x14ac:dyDescent="0.45">
+    <row r="45" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C45" s="30"/>
       <c r="D45" s="31"/>
       <c r="E45" s="31"/>
@@ -20006,6 +20006,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -20022,28 +20044,6 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">

</xml_diff>

<commit_message>
JRP Quali Zeitraum angepasst
</commit_message>
<xml_diff>
--- a/web/data/records_kriterien.xlsx
+++ b/web/data/records_kriterien.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB51B59-528E-4AEB-BE05-F671454C5529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FFC4FD5-4BF6-4F0F-8306-07D3A74B08D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="687" activeTab="9" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" activeTab="6" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
   <sheets>
     <sheet name="DR" sheetId="9" r:id="rId1"/>
@@ -754,12 +754,6 @@
     <t>200m Hindernisschwimmen</t>
   </si>
   <si>
-    <t>JRP (TEST) Weiblich</t>
-  </si>
-  <si>
-    <t>JRP (TEST) Männlich</t>
-  </si>
-  <si>
     <t>datum von</t>
   </si>
   <si>
@@ -1013,6 +1007,12 @@
   </si>
   <si>
     <t>1000</t>
+  </si>
+  <si>
+    <t>Richtzeiten Männlich</t>
+  </si>
+  <si>
+    <t>Richtzeiten Weiblich</t>
   </si>
 </sst>
 </file>
@@ -1701,13 +1701,16 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1719,6 +1722,15 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1727,6 +1739,27 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1770,39 +1803,6 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
@@ -1916,18 +1916,7 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="25" formatCode="hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="25" formatCode="hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1978,10 +1967,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2238,6 +2223,75 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -4287,73 +4341,19 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4369,102 +4369,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="212" headerRowBorderDxfId="211" tableBorderDxfId="210">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="230" headerRowBorderDxfId="229" tableBorderDxfId="228">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="209">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="227">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="208"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="207"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="206"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="205"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="204"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="203"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="202"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="201"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="226"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="225"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="224"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="223"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="222"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="221"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="220"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="219"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="200"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="199"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="198"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="197"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="196"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="195"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="194"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="193"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="192"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="191"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="190"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="189"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="188"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="187"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="186"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="185"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="184"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="183"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="182"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="181"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="180"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="179"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="178"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="177"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="176"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="175"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="174"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="173"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="172"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="171"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="170"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="169"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="168"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="167"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="166"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="165"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="164"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="218"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="217"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="216"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="215"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="214"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="213"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="212"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="211"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="210"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="209"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="208"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="207"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="206"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="205"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="204"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="203"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="202"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="201"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="200"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="199"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="198"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="197"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="196"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="195"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="194"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="193"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="192"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="191"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="190"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="189"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="188"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="187"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="186"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="185"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="184"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="183"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="182"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="163" dataDxfId="161" headerRowBorderDxfId="162" tableBorderDxfId="160">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="181" dataDxfId="179" headerRowBorderDxfId="180" tableBorderDxfId="178">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="159"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="158"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="157"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="156"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="155"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="154"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="153"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="152"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="151"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="150"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="149"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="148"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="147"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="177"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="176"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="175"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="174"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="173"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="172"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="171"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="170"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="169"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="168"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="167"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="166"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="165"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="146" headerRowBorderDxfId="145" tableBorderDxfId="144">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="164" headerRowBorderDxfId="163" tableBorderDxfId="162">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="143">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="161">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="142"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="141"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="140"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="139"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="138"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="137"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="136"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="135"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="160"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="159"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="158"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="157"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="156"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="155"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="154"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="153"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -4475,7 +4475,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="235" dataDxfId="234">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="152" dataDxfId="151">
   <autoFilter ref="A1:U3" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4500,64 +4500,64 @@
     <filterColumn colId="20" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="233"/>
-    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="232"/>
-    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="231"/>
-    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="230"/>
-    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="229"/>
-    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="228"/>
-    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="227"/>
-    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="226"/>
-    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="225"/>
-    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="224"/>
-    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="223"/>
-    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="222"/>
-    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="221"/>
-    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="220"/>
-    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="219"/>
-    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="218"/>
-    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="217"/>
-    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="216"/>
-    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="215"/>
-    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="214"/>
-    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="213"/>
+    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="150"/>
+    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="149"/>
+    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="148"/>
+    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="147"/>
+    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="146"/>
+    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="145"/>
+    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="144"/>
+    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="143"/>
+    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="142"/>
+    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="141"/>
+    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="140"/>
+    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="139"/>
+    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="138"/>
+    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="137"/>
+    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="136"/>
+    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="135"/>
+    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="134"/>
+    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="133"/>
+    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="132"/>
+    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="131"/>
+    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="130"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="134" dataDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:U7" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="132"/>
-    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="131"/>
-    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="130"/>
-    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="129"/>
-    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="128"/>
-    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="127"/>
-    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="126"/>
-    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="125"/>
-    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="124"/>
-    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="123"/>
-    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="122"/>
-    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="121"/>
-    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="120"/>
-    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="119"/>
-    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="118"/>
-    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="117"/>
-    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="116"/>
-    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="115"/>
-    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="114"/>
-    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="113"/>
-    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="112"/>
+    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="123"/>
+    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="122"/>
+    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="121"/>
+    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="120"/>
+    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="119"/>
+    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="118"/>
+    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="117"/>
+    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="116"/>
+    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="115"/>
+    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="114"/>
+    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="113"/>
+    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="112"/>
+    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="111"/>
+    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="110"/>
+    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="109"/>
+    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="108"/>
+    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="107"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
   <autoFilter ref="A1:X7" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4585,37 +4585,37 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="105"/>
-    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="104"/>
-    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="103"/>
-    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="102"/>
-    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="101"/>
-    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="100"/>
-    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="99"/>
-    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="98"/>
-    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="97"/>
-    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="96"/>
-    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="95"/>
-    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="94"/>
-    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="93"/>
-    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="92"/>
-    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="91"/>
-    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="90"/>
-    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="89"/>
-    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="88"/>
-    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="87"/>
-    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="86"/>
+    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="103"/>
+    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="102"/>
+    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="101"/>
+    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="100"/>
+    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="99"/>
+    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="98"/>
+    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="97"/>
+    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="96"/>
+    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="95"/>
+    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="94"/>
+    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="93"/>
+    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="92"/>
+    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="91"/>
+    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="90"/>
+    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="89"/>
+    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="88"/>
+    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="87"/>
+    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="86"/>
+    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="85"/>
+    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="84"/>
+    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="83"/>
+    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="82"/>
+    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
   <autoFilter ref="A1:X3" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4643,71 +4643,71 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="83"/>
-    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="82"/>
-    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="80"/>
-    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="79"/>
-    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="78"/>
-    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="77"/>
-    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="75"/>
-    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="74"/>
-    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="73"/>
-    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="72"/>
-    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="71"/>
-    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="70"/>
-    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="69"/>
-    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="68"/>
-    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="67"/>
-    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="66"/>
-    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="65"/>
-    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="64"/>
-    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="63"/>
-    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="62"/>
-    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="61"/>
-    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="71"/>
+    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="70"/>
+    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="69"/>
+    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="68"/>
+    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="67"/>
+    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="66"/>
+    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="65"/>
+    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="64"/>
+    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="63"/>
+    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="62"/>
+    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="61"/>
+    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="60"/>
+    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="59"/>
+    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="58"/>
+    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="57"/>
+    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="56"/>
+    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53">
   <autoFilter ref="A1:AF37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
   <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="52"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="50"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="48"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="46"/>
-    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="45"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="44"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="43"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="42"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="41"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="40"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="39"/>
-    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="38"/>
-    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="37"/>
-    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="36"/>
-    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="35"/>
-    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="34"/>
-    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="33"/>
-    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="32"/>
-    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="31"/>
-    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="30"/>
-    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="29"/>
-    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="28"/>
-    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="27"/>
-    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="41"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="40"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="39"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="38"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="37"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="36"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="35"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="34"/>
+    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="33"/>
+    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="32"/>
+    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="31"/>
+    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="30"/>
+    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="29"/>
+    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="28"/>
+    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="27"/>
+    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="26"/>
+    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="25"/>
+    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="24"/>
+    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="23"/>
+    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="22"/>
+    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4717,12 +4717,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}" name="LK_Kalender" displayName="LK_Kalender" ref="A1:H8" totalsRowShown="0">
   <autoFilter ref="A1:H8" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="235"/>
     <tableColumn id="2" xr3:uid="{38211212-0A92-428C-895C-E4CA68F52818}" name="datum bis"/>
-    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="234"/>
+    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="233"/>
+    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="232"/>
+    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="231"/>
     <tableColumn id="7" xr3:uid="{E7E62A34-7A76-4361-937D-F4DE76E6E7CC}" name="ort"/>
     <tableColumn id="8" xr3:uid="{84F02734-FC16-406B-ACCA-0CCDF547D94C}" name="kader"/>
   </tableColumns>
@@ -5049,9 +5049,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0519F5DB-31A0-4819-8E86-33B1F16466A6}">
   <sheetPr codeName="Tabelle6"/>
   <dimension ref="A1:AW31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.265625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
@@ -5120,7 +5120,7 @@
       <c r="AV1" s="10"/>
       <c r="AW1" s="10"/>
     </row>
-    <row r="2" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -5187,7 +5187,7 @@
       <c r="AV2" s="11"/>
       <c r="AW2" s="11"/>
     </row>
-    <row r="3" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>67</v>
       </c>
@@ -5248,7 +5248,7 @@
       <c r="AV3" s="11"/>
       <c r="AW3" s="11"/>
     </row>
-    <row r="4" spans="1:49" s="19" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:49" s="19" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
@@ -5397,7 +5397,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>2000</v>
       </c>
@@ -5450,7 +5450,7 @@
       <c r="AV5" s="3"/>
       <c r="AW5" s="3"/>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <f t="shared" ref="A6:A31" si="0">A5+1</f>
         <v>2001</v>
@@ -5528,7 +5528,7 @@
       <c r="AV6" s="4"/>
       <c r="AW6" s="4"/>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>2002</v>
@@ -5606,7 +5606,7 @@
       <c r="AV7" s="3"/>
       <c r="AW7" s="3"/>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>2003</v>
@@ -5684,7 +5684,7 @@
       <c r="AV8" s="4"/>
       <c r="AW8" s="4"/>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>2004</v>
@@ -5762,7 +5762,7 @@
       <c r="AV9" s="3"/>
       <c r="AW9" s="3"/>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>2005</v>
@@ -5840,7 +5840,7 @@
       <c r="AV10" s="4"/>
       <c r="AW10" s="4"/>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>2006</v>
@@ -5918,7 +5918,7 @@
       <c r="AV11" s="3"/>
       <c r="AW11" s="3"/>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>2007</v>
@@ -6040,7 +6040,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>2008</v>
@@ -6162,7 +6162,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>2009</v>
@@ -6284,7 +6284,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>2010</v>
@@ -6406,7 +6406,7 @@
         <v>3.5995370370370369E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>2011</v>
@@ -6540,7 +6540,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <f t="shared" si="0"/>
         <v>2012</v>
@@ -6674,7 +6674,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
         <v>2013</v>
@@ -6808,7 +6808,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <f t="shared" si="0"/>
         <v>2014</v>
@@ -6942,7 +6942,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <f t="shared" si="0"/>
         <v>2015</v>
@@ -7076,7 +7076,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
         <f t="shared" si="0"/>
         <v>2016</v>
@@ -7210,7 +7210,7 @@
         <v>3.5324074074074077E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
         <f t="shared" si="0"/>
         <v>2017</v>
@@ -7344,7 +7344,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
         <f t="shared" si="0"/>
         <v>2018</v>
@@ -7478,7 +7478,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
         <f t="shared" si="0"/>
         <v>2019</v>
@@ -7612,7 +7612,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
         <f t="shared" si="0"/>
         <v>2020</v>
@@ -7762,7 +7762,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
         <f t="shared" si="0"/>
         <v>2021</v>
@@ -7912,7 +7912,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
         <f t="shared" si="0"/>
         <v>2022</v>
@@ -8062,7 +8062,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -8212,7 +8212,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -8362,7 +8362,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -8512,7 +8512,7 @@
         <v>3.4745370370370372E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A31" s="1">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -8728,44 +8728,44 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="84.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="84.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.73046875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C1" t="s">
         <v>191</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>192</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>193</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>199</v>
+      </c>
+      <c r="G1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H1" t="s">
         <v>194</v>
       </c>
-      <c r="E1" t="s">
-        <v>195</v>
-      </c>
-      <c r="F1" t="s">
-        <v>201</v>
-      </c>
-      <c r="G1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H1" t="s">
-        <v>196</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" s="36">
         <v>46124</v>
       </c>
@@ -8776,19 +8776,19 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="E2" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="F2" s="38" t="s">
+        <v>200</v>
+      </c>
+      <c r="G2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H2" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="38" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" t="s">
-        <v>199</v>
-      </c>
-      <c r="H2" t="s">
-        <v>200</v>
-      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" s="36">
         <v>46124</v>
       </c>
@@ -8799,19 +8799,19 @@
         <v>0.65625</v>
       </c>
       <c r="E3" s="38" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F3" s="38" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" s="36">
         <v>46186</v>
       </c>
@@ -8822,19 +8822,19 @@
         <v>0.76041666666666663</v>
       </c>
       <c r="E4" s="38" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="38" t="s">
         <v>203</v>
       </c>
-      <c r="F4" s="38" t="s">
-        <v>205</v>
-      </c>
       <c r="G4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" s="36">
         <v>46187</v>
       </c>
@@ -8845,19 +8845,19 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="E5" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="F5" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="G5" t="s">
+        <v>197</v>
+      </c>
+      <c r="H5" t="s">
         <v>198</v>
       </c>
-      <c r="F5" s="38" t="s">
-        <v>207</v>
-      </c>
-      <c r="G5" t="s">
-        <v>199</v>
-      </c>
-      <c r="H5" t="s">
-        <v>200</v>
-      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" s="36">
         <v>46199</v>
       </c>
@@ -8871,19 +8871,19 @@
         <v>0.99930555555555556</v>
       </c>
       <c r="E6" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="G6" t="s">
         <v>208</v>
       </c>
-      <c r="F6" s="38" t="s">
-        <v>209</v>
-      </c>
-      <c r="G6" t="s">
-        <v>210</v>
-      </c>
       <c r="H6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" s="36">
         <v>46201</v>
       </c>
@@ -8894,19 +8894,19 @@
         <v>0.75</v>
       </c>
       <c r="E7" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>236</v>
+      </c>
+      <c r="G7" t="s">
+        <v>210</v>
+      </c>
+      <c r="H7" t="s">
         <v>211</v>
       </c>
-      <c r="F7" s="38" t="s">
-        <v>238</v>
-      </c>
-      <c r="G7" t="s">
-        <v>212</v>
-      </c>
-      <c r="H7" t="s">
-        <v>213</v>
-      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" s="36">
         <v>46228</v>
       </c>
@@ -8917,16 +8917,16 @@
         <v>0.99930555555555556</v>
       </c>
       <c r="E8" s="38" t="s">
+        <v>212</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>213</v>
+      </c>
+      <c r="G8" t="s">
         <v>214</v>
       </c>
-      <c r="F8" s="38" t="s">
+      <c r="H8" t="s">
         <v>215</v>
-      </c>
-      <c r="G8" t="s">
-        <v>216</v>
-      </c>
-      <c r="H8" t="s">
-        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -8946,17 +8946,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB2B168-68B3-410F-B4A6-8D511F9C32E0}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" customWidth="1"/>
-    <col min="2" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" customWidth="1"/>
-    <col min="7" max="11" width="18.7109375" customWidth="1"/>
-    <col min="12" max="12" width="22.140625" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.265625" customWidth="1"/>
+    <col min="2" max="5" width="18.73046875" customWidth="1"/>
+    <col min="6" max="6" width="21.1328125" customWidth="1"/>
+    <col min="7" max="11" width="18.73046875" customWidth="1"/>
+    <col min="12" max="12" width="22.1328125" customWidth="1"/>
+    <col min="13" max="13" width="18.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -9038,7 +9038,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>15</v>
       </c>
@@ -9079,7 +9079,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -9120,7 +9120,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>2000</v>
       </c>
@@ -9137,7 +9137,7 @@
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <f t="shared" ref="A6:A32" si="0">A5+1</f>
         <v>2001</v>
@@ -9155,7 +9155,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>2002</v>
@@ -9173,7 +9173,7 @@
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>2003</v>
@@ -9191,7 +9191,7 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>2004</v>
@@ -9209,7 +9209,7 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>2005</v>
@@ -9227,7 +9227,7 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>2006</v>
@@ -9245,7 +9245,7 @@
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>2007</v>
@@ -9263,7 +9263,7 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>2008</v>
@@ -9281,7 +9281,7 @@
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>2009</v>
@@ -9299,7 +9299,7 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>2010</v>
@@ -9317,7 +9317,7 @@
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>2011</v>
@@ -9335,7 +9335,7 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <f t="shared" si="0"/>
         <v>2012</v>
@@ -9353,7 +9353,7 @@
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
         <v>2013</v>
@@ -9371,7 +9371,7 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <f t="shared" si="0"/>
         <v>2014</v>
@@ -9389,7 +9389,7 @@
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <f t="shared" si="0"/>
         <v>2015</v>
@@ -9431,7 +9431,7 @@
         <v>1.3592592592592591E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
         <f t="shared" si="0"/>
         <v>2016</v>
@@ -9473,7 +9473,7 @@
         <v>1.3592592592592591E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
         <f t="shared" si="0"/>
         <v>2017</v>
@@ -9515,7 +9515,7 @@
         <v>1.3577546296296298E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
         <f t="shared" si="0"/>
         <v>2018</v>
@@ -9557,7 +9557,7 @@
         <v>1.3577546296296298E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
         <f t="shared" si="0"/>
         <v>2019</v>
@@ -9599,7 +9599,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
         <f t="shared" si="0"/>
         <v>2020</v>
@@ -9641,7 +9641,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
         <f t="shared" si="0"/>
         <v>2021</v>
@@ -9683,7 +9683,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
         <f t="shared" si="0"/>
         <v>2022</v>
@@ -9725,7 +9725,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -9767,7 +9767,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -9809,7 +9809,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -9851,7 +9851,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="1">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -9893,7 +9893,7 @@
         <v>1.3511574074074075E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" s="1">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -9968,17 +9968,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC5FFB6C-7DEA-4C95-82B5-1769BD3934D8}">
   <sheetPr codeName="Tabelle2"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
-    <col min="2" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" customWidth="1"/>
-    <col min="7" max="11" width="18.7109375" customWidth="1"/>
-    <col min="12" max="12" width="22.140625" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.86328125" customWidth="1"/>
+    <col min="2" max="5" width="18.73046875" customWidth="1"/>
+    <col min="6" max="6" width="21.1328125" customWidth="1"/>
+    <col min="7" max="11" width="18.73046875" customWidth="1"/>
+    <col min="12" max="12" width="22.1328125" customWidth="1"/>
+    <col min="13" max="13" width="18.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
@@ -10019,7 +10019,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -10060,7 +10060,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>15</v>
       </c>
@@ -10101,7 +10101,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -10142,7 +10142,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>2000</v>
       </c>
@@ -10159,7 +10159,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <f t="shared" ref="A6:A31" si="0">A5+1</f>
         <v>2001</v>
@@ -10189,7 +10189,7 @@
         <v>1.3629629629629632E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>2002</v>
@@ -10231,7 +10231,7 @@
         <v>1.3629629629629632E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>2003</v>
@@ -10273,7 +10273,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>2004</v>
@@ -10315,7 +10315,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>2005</v>
@@ -10357,7 +10357,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>2006</v>
@@ -10399,7 +10399,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>2007</v>
@@ -10441,7 +10441,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>2008</v>
@@ -10483,7 +10483,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>2009</v>
@@ -10525,7 +10525,7 @@
         <v>1.3346064814814815E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>2010</v>
@@ -10567,7 +10567,7 @@
         <v>1.3306712962962966E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>2011</v>
@@ -10609,7 +10609,7 @@
         <v>1.3306712962962966E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <f t="shared" si="0"/>
         <v>2012</v>
@@ -10651,7 +10651,7 @@
         <v>1.3306712962962966E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
         <v>2013</v>
@@ -10693,7 +10693,7 @@
         <v>1.312962962962963E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <f t="shared" si="0"/>
         <v>2014</v>
@@ -10735,7 +10735,7 @@
         <v>1.312962962962963E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <f t="shared" si="0"/>
         <v>2015</v>
@@ -10777,7 +10777,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
         <f t="shared" si="0"/>
         <v>2016</v>
@@ -10819,7 +10819,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
         <f t="shared" si="0"/>
         <v>2017</v>
@@ -10861,7 +10861,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
         <f t="shared" si="0"/>
         <v>2018</v>
@@ -10903,7 +10903,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
         <f t="shared" si="0"/>
         <v>2019</v>
@@ -10945,7 +10945,7 @@
         <v>1.3116898148148148E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
         <f t="shared" si="0"/>
         <v>2020</v>
@@ -10987,7 +10987,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
         <f t="shared" si="0"/>
         <v>2021</v>
@@ -11029,7 +11029,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
         <f t="shared" si="0"/>
         <v>2022</v>
@@ -11071,7 +11071,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -11113,7 +11113,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -11155,7 +11155,7 @@
         <v>1.3097222222222223E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -11197,7 +11197,7 @@
         <v>1.2931712962962962E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="1">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -11239,7 +11239,7 @@
         <v>1.2931712962962962E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" s="1">
         <f>A31+1</f>
         <v>2027</v>
@@ -11316,30 +11316,30 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:U3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" customWidth="1"/>
+    <col min="13" max="13" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.73046875" customWidth="1"/>
     <col min="15" max="16" width="19" customWidth="1"/>
-    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="22.265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="47.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="26" t="s">
         <v>127</v>
       </c>
@@ -11404,7 +11404,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
         <v>163</v>
       </c>
@@ -11461,7 +11461,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
         <v>164</v>
       </c>
@@ -11532,30 +11532,30 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:U7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" customWidth="1"/>
+    <col min="13" max="13" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.73046875" customWidth="1"/>
     <col min="15" max="16" width="19" customWidth="1"/>
-    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="22.265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="47.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="26" t="s">
         <v>127</v>
       </c>
@@ -11620,7 +11620,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
         <v>155</v>
       </c>
@@ -11634,7 +11634,7 @@
         <v>50</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F2" s="25" t="s">
         <v>161</v>
@@ -11681,7 +11681,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
         <v>156</v>
       </c>
@@ -11695,7 +11695,7 @@
         <v>50</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F3" s="25" t="s">
         <v>161</v>
@@ -11742,7 +11742,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A4" s="25" t="s">
         <v>157</v>
       </c>
@@ -11756,7 +11756,7 @@
         <v>18</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F4" s="25" t="s">
         <v>161</v>
@@ -11800,10 +11800,10 @@
         <v>10</v>
       </c>
       <c r="U4" s="25" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A5" s="25" t="s">
         <v>158</v>
       </c>
@@ -11817,7 +11817,7 @@
         <v>18</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F5" s="25" t="s">
         <v>161</v>
@@ -11862,7 +11862,7 @@
       </c>
       <c r="U5" s="25"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A6" s="25" t="s">
         <v>159</v>
       </c>
@@ -11876,7 +11876,7 @@
         <v>16</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F6" s="25" t="s">
         <v>161</v>
@@ -11921,7 +11921,7 @@
       </c>
       <c r="U6" s="25"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A7" s="25" t="s">
         <v>160</v>
       </c>
@@ -11935,7 +11935,7 @@
         <v>16</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F7" s="25" t="s">
         <v>161</v>
@@ -11994,35 +11994,35 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:X7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.3984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.86328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12096,7 +12096,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
         <v>178</v>
       </c>
@@ -12166,7 +12166,7 @@
         <v>1.9623842592592592E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
         <v>179</v>
       </c>
@@ -12236,7 +12236,7 @@
         <v>1.8121527777777778E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A4" s="25" t="s">
         <v>180</v>
       </c>
@@ -12306,7 +12306,7 @@
         <v>1.9979166666666665E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A5" s="25" t="s">
         <v>181</v>
       </c>
@@ -12376,7 +12376,7 @@
         <v>1.7653935185185186E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A6" s="25" t="s">
         <v>155</v>
       </c>
@@ -12446,7 +12446,7 @@
         <v>1.8998842592592594E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A7" s="25" t="s">
         <v>156</v>
       </c>
@@ -12530,35 +12530,35 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:X3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.86328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.73046875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.86328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.59765625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="27" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="22" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.59765625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12632,9 +12632,9 @@
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
-        <v>189</v>
+        <v>275</v>
       </c>
       <c r="B2" s="25" t="s">
         <v>130</v>
@@ -12646,13 +12646,13 @@
         <v>18</v>
       </c>
       <c r="E2" s="27">
-        <v>45658</v>
+        <v>45839</v>
       </c>
       <c r="F2" s="27">
-        <v>46174</v>
+        <v>46193</v>
       </c>
       <c r="G2" s="27">
-        <v>45658</v>
+        <v>46023</v>
       </c>
       <c r="H2" s="25" t="s">
         <v>144</v>
@@ -12702,9 +12702,9 @@
         <v>1.8332175925925925E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
-        <v>190</v>
+        <v>274</v>
       </c>
       <c r="B3" s="25" t="s">
         <v>148</v>
@@ -12716,13 +12716,13 @@
         <v>18</v>
       </c>
       <c r="E3" s="27">
-        <v>45658</v>
+        <v>45839</v>
       </c>
       <c r="F3" s="27">
-        <v>46174</v>
+        <v>46193</v>
       </c>
       <c r="G3" s="27">
-        <v>45658</v>
+        <v>46023</v>
       </c>
       <c r="H3" s="25" t="s">
         <v>144</v>
@@ -12786,30 +12786,30 @@
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AF37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.3984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.3984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.86328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.1328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A1" s="25" t="s">
         <v>127</v>
       </c>
@@ -12847,69 +12847,69 @@
         <v>142</v>
       </c>
       <c r="M1" s="25" t="s">
+        <v>245</v>
+      </c>
+      <c r="N1" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="O1" s="25" t="s">
         <v>247</v>
       </c>
-      <c r="N1" s="25" t="s">
+      <c r="P1" s="25" t="s">
         <v>248</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="Q1" s="25" t="s">
         <v>249</v>
       </c>
-      <c r="P1" s="25" t="s">
+      <c r="R1" s="25" t="s">
         <v>250</v>
       </c>
-      <c r="Q1" s="25" t="s">
+      <c r="S1" s="25" t="s">
         <v>251</v>
       </c>
-      <c r="R1" s="25" t="s">
+      <c r="T1" s="25" t="s">
         <v>252</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="U1" s="25" t="s">
         <v>253</v>
       </c>
-      <c r="T1" s="25" t="s">
+      <c r="V1" s="25" t="s">
         <v>254</v>
       </c>
-      <c r="U1" s="25" t="s">
+      <c r="W1" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="X1" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="Y1" s="25" t="s">
+        <v>262</v>
+      </c>
+      <c r="Z1" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="V1" s="25" t="s">
-        <v>256</v>
-      </c>
-      <c r="W1" s="25" t="s">
+      <c r="AA1" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="AB1" s="25" t="s">
+        <v>264</v>
+      </c>
+      <c r="AC1" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="AD1" s="25" t="s">
         <v>258</v>
       </c>
-      <c r="X1" s="25" t="s">
-        <v>263</v>
-      </c>
-      <c r="Y1" s="25" t="s">
-        <v>264</v>
-      </c>
-      <c r="Z1" s="25" t="s">
-        <v>257</v>
-      </c>
-      <c r="AA1" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="AB1" s="25" t="s">
-        <v>266</v>
-      </c>
-      <c r="AC1" s="25" t="s">
+      <c r="AE1" s="25" t="s">
         <v>259</v>
       </c>
-      <c r="AD1" s="25" t="s">
+      <c r="AF1" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="AE1" s="25" t="s">
-        <v>261</v>
-      </c>
-      <c r="AF1" s="25" t="s">
-        <v>262</v>
-      </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A2" s="25" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B2" s="25" t="s">
         <v>130</v>
@@ -12981,9 +12981,9 @@
       <c r="AE2" s="106"/>
       <c r="AF2" s="106"/>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A3" s="25" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B3" s="25" t="s">
         <v>130</v>
@@ -13055,9 +13055,9 @@
       <c r="AE3" s="106"/>
       <c r="AF3" s="106"/>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A4" s="25" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B4" s="25" t="s">
         <v>130</v>
@@ -13129,9 +13129,9 @@
       <c r="AE4" s="106"/>
       <c r="AF4" s="106"/>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A5" s="25" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B5" s="25" t="s">
         <v>148</v>
@@ -13203,9 +13203,9 @@
       <c r="AE5" s="106"/>
       <c r="AF5" s="106"/>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A6" s="25" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>148</v>
@@ -13277,9 +13277,9 @@
       <c r="AE6" s="106"/>
       <c r="AF6" s="106"/>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A7" s="25" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B7" s="25" t="s">
         <v>148</v>
@@ -13351,9 +13351,9 @@
       <c r="AE7" s="106"/>
       <c r="AF7" s="106"/>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A8" s="25" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B8" s="25" t="s">
         <v>130</v>
@@ -13425,9 +13425,9 @@
       <c r="AE8" s="106"/>
       <c r="AF8" s="106"/>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A9" s="25" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B9" s="25" t="s">
         <v>130</v>
@@ -13499,9 +13499,9 @@
       <c r="AE9" s="106"/>
       <c r="AF9" s="106"/>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A10" s="25" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B10" s="25" t="s">
         <v>130</v>
@@ -13573,9 +13573,9 @@
       <c r="AE10" s="106"/>
       <c r="AF10" s="106"/>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A11" s="25" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B11" s="25" t="s">
         <v>148</v>
@@ -13647,9 +13647,9 @@
       <c r="AE11" s="106"/>
       <c r="AF11" s="106"/>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A12" s="25" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B12" s="25" t="s">
         <v>148</v>
@@ -13721,9 +13721,9 @@
       <c r="AE12" s="106"/>
       <c r="AF12" s="106"/>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A13" s="25" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B13" s="25" t="s">
         <v>148</v>
@@ -13795,9 +13795,9 @@
       <c r="AE13" s="106"/>
       <c r="AF13" s="106"/>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A14" s="25" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B14" s="25" t="s">
         <v>130</v>
@@ -13862,28 +13862,28 @@
       <c r="V14" s="106"/>
       <c r="W14" s="106"/>
       <c r="X14" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y14" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z14" s="106" t="s">
         <v>272</v>
-      </c>
-      <c r="Y14" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z14" s="106" t="s">
-        <v>274</v>
       </c>
       <c r="AA14" s="106"/>
       <c r="AB14" s="106"/>
       <c r="AC14" s="106"/>
       <c r="AD14" s="106"/>
       <c r="AE14" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AF14" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A15" s="25" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B15" s="25" t="s">
         <v>130</v>
@@ -13945,33 +13945,33 @@
       </c>
       <c r="T15" s="106"/>
       <c r="U15" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V15" s="106"/>
       <c r="W15" s="106"/>
       <c r="X15" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y15" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z15" s="106" t="s">
         <v>272</v>
-      </c>
-      <c r="Y15" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z15" s="106" t="s">
-        <v>274</v>
       </c>
       <c r="AA15" s="106"/>
       <c r="AB15" s="106"/>
       <c r="AC15" s="106"/>
       <c r="AD15" s="106"/>
       <c r="AE15" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AF15" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A16" s="25" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B16" s="25" t="s">
         <v>130</v>
@@ -14033,33 +14033,33 @@
       </c>
       <c r="T16" s="106"/>
       <c r="U16" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V16" s="106"/>
       <c r="W16" s="106"/>
       <c r="X16" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y16" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z16" s="106" t="s">
         <v>272</v>
-      </c>
-      <c r="Y16" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z16" s="106" t="s">
-        <v>274</v>
       </c>
       <c r="AA16" s="106"/>
       <c r="AB16" s="106"/>
       <c r="AC16" s="106"/>
       <c r="AD16" s="106"/>
       <c r="AE16" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AF16" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A17" s="25" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B17" s="25" t="s">
         <v>148</v>
@@ -14124,28 +14124,28 @@
       <c r="V17" s="106"/>
       <c r="W17" s="106"/>
       <c r="X17" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y17" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z17" s="106" t="s">
         <v>272</v>
-      </c>
-      <c r="Y17" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z17" s="106" t="s">
-        <v>274</v>
       </c>
       <c r="AA17" s="106"/>
       <c r="AB17" s="106"/>
       <c r="AC17" s="106"/>
       <c r="AD17" s="106"/>
       <c r="AE17" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AF17" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A18" s="25" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>148</v>
@@ -14207,33 +14207,33 @@
       </c>
       <c r="T18" s="106"/>
       <c r="U18" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V18" s="106"/>
       <c r="W18" s="106"/>
       <c r="X18" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y18" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z18" s="106" t="s">
         <v>272</v>
-      </c>
-      <c r="Y18" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z18" s="106" t="s">
-        <v>274</v>
       </c>
       <c r="AA18" s="106"/>
       <c r="AB18" s="106"/>
       <c r="AC18" s="106"/>
       <c r="AD18" s="106"/>
       <c r="AE18" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AF18" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A19" s="25" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>148</v>
@@ -14295,33 +14295,33 @@
       </c>
       <c r="T19" s="106"/>
       <c r="U19" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V19" s="106"/>
       <c r="W19" s="106"/>
       <c r="X19" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="Y19" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="Z19" s="106" t="s">
         <v>272</v>
-      </c>
-      <c r="Y19" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z19" s="106" t="s">
-        <v>274</v>
       </c>
       <c r="AA19" s="106"/>
       <c r="AB19" s="106"/>
       <c r="AC19" s="106"/>
       <c r="AD19" s="106"/>
       <c r="AE19" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AF19" s="106" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A20" s="25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B20" s="25" t="s">
         <v>130</v>
@@ -14386,28 +14386,28 @@
       <c r="V20" s="106"/>
       <c r="W20" s="106"/>
       <c r="X20" s="106" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="Y20" s="106" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="Z20" s="106"/>
       <c r="AA20" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB20" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="AC20" s="106"/>
       <c r="AD20" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AE20" s="106"/>
       <c r="AF20" s="106"/>
     </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A21" s="25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B21" s="25" t="s">
         <v>130</v>
@@ -14472,28 +14472,28 @@
       <c r="V21" s="106"/>
       <c r="W21" s="106"/>
       <c r="X21" s="106" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="Y21" s="106" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="Z21" s="106"/>
       <c r="AA21" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB21" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="AC21" s="106"/>
       <c r="AD21" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AE21" s="106"/>
       <c r="AF21" s="106"/>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A22" s="25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B22" s="25" t="s">
         <v>130</v>
@@ -14555,35 +14555,35 @@
       </c>
       <c r="T22" s="106"/>
       <c r="U22" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V22" s="106"/>
       <c r="W22" s="106"/>
       <c r="X22" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y22" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z22" s="106"/>
       <c r="AA22" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB22" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AC22" s="106"/>
       <c r="AD22" s="106"/>
       <c r="AE22" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AF22" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A23" s="25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B23" s="25" t="s">
         <v>130</v>
@@ -14645,35 +14645,35 @@
       </c>
       <c r="T23" s="106"/>
       <c r="U23" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V23" s="106"/>
       <c r="W23" s="106"/>
       <c r="X23" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y23" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z23" s="106"/>
       <c r="AA23" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB23" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AC23" s="106"/>
       <c r="AD23" s="106"/>
       <c r="AE23" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AF23" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A24" s="25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B24" s="25" t="s">
         <v>130</v>
@@ -14738,30 +14738,30 @@
       <c r="V24" s="106"/>
       <c r="W24" s="106"/>
       <c r="X24" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y24" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z24" s="106"/>
       <c r="AA24" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB24" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AC24" s="106"/>
       <c r="AD24" s="106"/>
       <c r="AE24" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AF24" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A25" s="25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B25" s="25" t="s">
         <v>148</v>
@@ -14826,28 +14826,28 @@
       <c r="V25" s="106"/>
       <c r="W25" s="106"/>
       <c r="X25" s="106" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="Y25" s="106" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="Z25" s="106"/>
       <c r="AA25" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB25" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="AC25" s="106"/>
       <c r="AD25" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AE25" s="106"/>
       <c r="AF25" s="106"/>
     </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A26" s="25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B26" s="25" t="s">
         <v>148</v>
@@ -14912,28 +14912,28 @@
       <c r="V26" s="106"/>
       <c r="W26" s="106"/>
       <c r="X26" s="106" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="Y26" s="106" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="Z26" s="106"/>
       <c r="AA26" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB26" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="AC26" s="106"/>
       <c r="AD26" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AE26" s="106"/>
       <c r="AF26" s="106"/>
     </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A27" s="25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B27" s="25" t="s">
         <v>148</v>
@@ -14995,35 +14995,35 @@
       </c>
       <c r="T27" s="106"/>
       <c r="U27" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V27" s="106"/>
       <c r="W27" s="106"/>
       <c r="X27" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y27" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z27" s="106"/>
       <c r="AA27" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB27" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AC27" s="106"/>
       <c r="AD27" s="106"/>
       <c r="AE27" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AF27" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A28" s="25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B28" s="25" t="s">
         <v>148</v>
@@ -15085,35 +15085,35 @@
       </c>
       <c r="T28" s="106"/>
       <c r="U28" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="V28" s="106"/>
       <c r="W28" s="106"/>
       <c r="X28" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y28" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z28" s="106"/>
       <c r="AA28" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB28" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AC28" s="106"/>
       <c r="AD28" s="106"/>
       <c r="AE28" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AF28" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A29" s="25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B29" s="25" t="s">
         <v>148</v>
@@ -15178,30 +15178,30 @@
       <c r="V29" s="106"/>
       <c r="W29" s="106"/>
       <c r="X29" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y29" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z29" s="106"/>
       <c r="AA29" s="106" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB29" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AC29" s="106"/>
       <c r="AD29" s="106"/>
       <c r="AE29" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AF29" s="106" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A30" s="25" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B30" s="25" t="s">
         <v>130</v>
@@ -15266,28 +15266,28 @@
       <c r="V30" s="106"/>
       <c r="W30" s="106"/>
       <c r="X30" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y30" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z30" s="106"/>
       <c r="AA30" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB30" s="106"/>
       <c r="AC30" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD30" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE30" s="106"/>
       <c r="AF30" s="106"/>
     </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A31" s="25" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B31" s="25" t="s">
         <v>130</v>
@@ -15352,28 +15352,28 @@
       <c r="V31" s="106"/>
       <c r="W31" s="106"/>
       <c r="X31" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y31" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z31" s="106"/>
       <c r="AA31" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB31" s="106"/>
       <c r="AC31" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD31" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE31" s="106"/>
       <c r="AF31" s="106"/>
     </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A32" s="25" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B32" s="25" t="s">
         <v>130</v>
@@ -15438,28 +15438,28 @@
       <c r="V32" s="106"/>
       <c r="W32" s="106"/>
       <c r="X32" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y32" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z32" s="106"/>
       <c r="AA32" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB32" s="106"/>
       <c r="AC32" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD32" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE32" s="106"/>
       <c r="AF32" s="106"/>
     </row>
-    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A33" s="25" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B33" s="25" t="s">
         <v>130</v>
@@ -15524,28 +15524,28 @@
       <c r="V33" s="106"/>
       <c r="W33" s="106"/>
       <c r="X33" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y33" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z33" s="106"/>
       <c r="AA33" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB33" s="106"/>
       <c r="AC33" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD33" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE33" s="106"/>
       <c r="AF33" s="106"/>
     </row>
-    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A34" s="25" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B34" s="25" t="s">
         <v>148</v>
@@ -15610,28 +15610,28 @@
       <c r="V34" s="106"/>
       <c r="W34" s="106"/>
       <c r="X34" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y34" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z34" s="106"/>
       <c r="AA34" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB34" s="106"/>
       <c r="AC34" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD34" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE34" s="106"/>
       <c r="AF34" s="106"/>
     </row>
-    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A35" s="25" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B35" s="25" t="s">
         <v>148</v>
@@ -15696,28 +15696,28 @@
       <c r="V35" s="106"/>
       <c r="W35" s="106"/>
       <c r="X35" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y35" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z35" s="106"/>
       <c r="AA35" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB35" s="106"/>
       <c r="AC35" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD35" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE35" s="106"/>
       <c r="AF35" s="106"/>
     </row>
-    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A36" s="25" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B36" s="25" t="s">
         <v>148</v>
@@ -15782,28 +15782,28 @@
       <c r="V36" s="106"/>
       <c r="W36" s="106"/>
       <c r="X36" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y36" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z36" s="106"/>
       <c r="AA36" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB36" s="106"/>
       <c r="AC36" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD36" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE36" s="106"/>
       <c r="AF36" s="106"/>
     </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A37" s="25" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B37" s="25" t="s">
         <v>148</v>
@@ -15868,21 +15868,21 @@
       <c r="V37" s="106"/>
       <c r="W37" s="106"/>
       <c r="X37" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y37" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="Z37" s="106"/>
       <c r="AA37" s="106" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AB37" s="106"/>
       <c r="AC37" s="106" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AD37" s="106" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AE37" s="106"/>
       <c r="AF37" s="106"/>
@@ -15900,147 +15900,147 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A13DA696-49DD-4BFA-98FE-5C7770404E50}">
   <sheetPr codeName="Tabelle12"/>
   <dimension ref="A1:BZ45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" customWidth="1"/>
-    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="26" width="9.5703125" customWidth="1"/>
-    <col min="28" max="28" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="52" width="4.5703125" customWidth="1"/>
-    <col min="54" max="54" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="55" max="78" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="5.265625" customWidth="1"/>
+    <col min="2" max="2" width="32.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="26" width="9.59765625" customWidth="1"/>
+    <col min="28" max="28" width="32.3984375" bestFit="1" customWidth="1"/>
+    <col min="29" max="52" width="4.59765625" customWidth="1"/>
+    <col min="54" max="54" width="32.3984375" bestFit="1" customWidth="1"/>
+    <col min="55" max="78" width="9.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="107">
+    <row r="1" spans="1:78" s="40" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="126">
         <v>2025</v>
       </c>
       <c r="B1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="108" t="s">
+      <c r="C1" s="107" t="s">
+        <v>218</v>
+      </c>
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="111" t="s">
+        <v>219</v>
+      </c>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="117" t="s">
+        <v>223</v>
+      </c>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="109" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="108"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="110" t="s">
+      <c r="P1" s="109"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="123" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="113" t="s">
-        <v>225</v>
-      </c>
-      <c r="L1" s="114"/>
-      <c r="M1" s="114"/>
-      <c r="N1" s="115"/>
-      <c r="O1" s="133" t="s">
-        <v>222</v>
-      </c>
-      <c r="P1" s="133"/>
-      <c r="Q1" s="134"/>
-      <c r="R1" s="135" t="s">
-        <v>223</v>
-      </c>
-      <c r="S1" s="136"/>
-      <c r="T1" s="136"/>
-      <c r="U1" s="136"/>
-      <c r="V1" s="137"/>
-      <c r="W1" s="138" t="s">
-        <v>226</v>
-      </c>
-      <c r="X1" s="139"/>
-      <c r="Y1" s="139"/>
-      <c r="Z1" s="140"/>
+      <c r="S1" s="124"/>
+      <c r="T1" s="124"/>
+      <c r="U1" s="124"/>
+      <c r="V1" s="125"/>
+      <c r="W1" s="120" t="s">
+        <v>224</v>
+      </c>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="122"/>
       <c r="AA1"/>
       <c r="AB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="116" t="s">
+      <c r="AC1" s="127" t="s">
+        <v>225</v>
+      </c>
+      <c r="AD1" s="127"/>
+      <c r="AE1" s="128"/>
+      <c r="AF1" s="129" t="s">
+        <v>226</v>
+      </c>
+      <c r="AG1" s="130"/>
+      <c r="AH1" s="130"/>
+      <c r="AI1" s="130"/>
+      <c r="AJ1" s="131"/>
+      <c r="AK1" s="132" t="s">
         <v>227</v>
       </c>
-      <c r="AD1" s="116"/>
-      <c r="AE1" s="117"/>
-      <c r="AF1" s="118" t="s">
+      <c r="AL1" s="133"/>
+      <c r="AM1" s="133"/>
+      <c r="AN1" s="134"/>
+      <c r="AO1" s="135" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="119"/>
-      <c r="AH1" s="119"/>
-      <c r="AI1" s="119"/>
-      <c r="AJ1" s="120"/>
-      <c r="AK1" s="121" t="s">
+      <c r="AP1" s="136"/>
+      <c r="AQ1" s="137"/>
+      <c r="AR1" s="138" t="s">
         <v>229</v>
       </c>
-      <c r="AL1" s="122"/>
-      <c r="AM1" s="122"/>
-      <c r="AN1" s="123"/>
-      <c r="AO1" s="124" t="s">
+      <c r="AS1" s="139"/>
+      <c r="AT1" s="139"/>
+      <c r="AU1" s="139"/>
+      <c r="AV1" s="140"/>
+      <c r="AW1" s="114" t="s">
         <v>230</v>
       </c>
-      <c r="AP1" s="125"/>
-      <c r="AQ1" s="126"/>
-      <c r="AR1" s="127" t="s">
-        <v>231</v>
-      </c>
-      <c r="AS1" s="128"/>
-      <c r="AT1" s="128"/>
-      <c r="AU1" s="128"/>
-      <c r="AV1" s="129"/>
-      <c r="AW1" s="130" t="s">
-        <v>232</v>
-      </c>
-      <c r="AX1" s="131"/>
-      <c r="AY1" s="131"/>
-      <c r="AZ1" s="132"/>
+      <c r="AX1" s="115"/>
+      <c r="AY1" s="115"/>
+      <c r="AZ1" s="116"/>
       <c r="BB1" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="108" t="s">
+      <c r="BC1" s="107" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD1" s="107"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="111" t="s">
+        <v>232</v>
+      </c>
+      <c r="BG1" s="112"/>
+      <c r="BH1" s="112"/>
+      <c r="BI1" s="112"/>
+      <c r="BJ1" s="113"/>
+      <c r="BK1" s="117" t="s">
         <v>233</v>
       </c>
-      <c r="BD1" s="108"/>
-      <c r="BE1" s="109"/>
-      <c r="BF1" s="110" t="s">
+      <c r="BL1" s="118"/>
+      <c r="BM1" s="118"/>
+      <c r="BN1" s="119"/>
+      <c r="BO1" s="109" t="s">
+        <v>239</v>
+      </c>
+      <c r="BP1" s="109"/>
+      <c r="BQ1" s="110"/>
+      <c r="BR1" s="123" t="s">
+        <v>240</v>
+      </c>
+      <c r="BS1" s="124"/>
+      <c r="BT1" s="124"/>
+      <c r="BU1" s="124"/>
+      <c r="BV1" s="125"/>
+      <c r="BW1" s="120" t="s">
         <v>234</v>
       </c>
-      <c r="BG1" s="111"/>
-      <c r="BH1" s="111"/>
-      <c r="BI1" s="111"/>
-      <c r="BJ1" s="112"/>
-      <c r="BK1" s="113" t="s">
-        <v>235</v>
-      </c>
-      <c r="BL1" s="114"/>
-      <c r="BM1" s="114"/>
-      <c r="BN1" s="115"/>
-      <c r="BO1" s="133" t="s">
-        <v>241</v>
-      </c>
-      <c r="BP1" s="133"/>
-      <c r="BQ1" s="134"/>
-      <c r="BR1" s="135" t="s">
-        <v>242</v>
-      </c>
-      <c r="BS1" s="136"/>
-      <c r="BT1" s="136"/>
-      <c r="BU1" s="136"/>
-      <c r="BV1" s="137"/>
-      <c r="BW1" s="138" t="s">
-        <v>236</v>
-      </c>
-      <c r="BX1" s="139"/>
-      <c r="BY1" s="139"/>
-      <c r="BZ1" s="140"/>
+      <c r="BX1" s="121"/>
+      <c r="BY1" s="121"/>
+      <c r="BZ1" s="122"/>
     </row>
-    <row r="2" spans="1:78" s="94" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="107"/>
+    <row r="2" spans="1:78" s="94" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="126"/>
       <c r="B2" s="46" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C2" s="41" t="str">
         <f ca="1">CONCATENATE("≤",YEAR(TODAY())-15-1)</f>
@@ -16140,7 +16140,7 @@
       </c>
       <c r="AA2"/>
       <c r="AB2" s="46" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="AC2" s="80" t="str">
         <f ca="1">CONCATENATE("≤",YEAR(TODAY())-15)</f>
@@ -16239,7 +16239,7 @@
         <v>2002-1986</v>
       </c>
       <c r="BB2" s="46" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="BC2" s="58" t="str">
         <f ca="1">CONCATENATE("≤",YEAR(TODAY())-15-1)</f>
@@ -16338,8 +16338,8 @@
         <v>2001-1985</v>
       </c>
     </row>
-    <row r="3" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="107"/>
+    <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="126"/>
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
@@ -16591,8 +16591,8 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A4" s="107"/>
+    <row r="4" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A4" s="126"/>
       <c r="B4" s="47" t="s">
         <v>185</v>
       </c>
@@ -16843,8 +16843,8 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A5" s="107"/>
+    <row r="5" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A5" s="126"/>
       <c r="B5" s="47" t="s">
         <v>186</v>
       </c>
@@ -17095,8 +17095,8 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A6" s="107"/>
+    <row r="6" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A6" s="126"/>
       <c r="B6" s="47" t="s">
         <v>187</v>
       </c>
@@ -17347,8 +17347,8 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A7" s="107"/>
+    <row r="7" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A7" s="126"/>
       <c r="B7" s="47" t="s">
         <v>188</v>
       </c>
@@ -17599,8 +17599,8 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:78" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="107"/>
+    <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A8" s="126"/>
       <c r="B8" s="50" t="s">
         <v>4</v>
       </c>
@@ -17851,136 +17851,136 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:78" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="107">
+    <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
+      <c r="A10" s="126">
         <v>2026</v>
       </c>
       <c r="B10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="108" t="s">
+      <c r="C10" s="107" t="s">
+        <v>218</v>
+      </c>
+      <c r="D10" s="107"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="111" t="s">
+        <v>219</v>
+      </c>
+      <c r="G10" s="112"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+      <c r="J10" s="113"/>
+      <c r="K10" s="117" t="s">
+        <v>223</v>
+      </c>
+      <c r="L10" s="118"/>
+      <c r="M10" s="118"/>
+      <c r="N10" s="119"/>
+      <c r="O10" s="109" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="108"/>
-      <c r="E10" s="109"/>
-      <c r="F10" s="110" t="s">
+      <c r="P10" s="109"/>
+      <c r="Q10" s="110"/>
+      <c r="R10" s="123" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="111"/>
-      <c r="H10" s="111"/>
-      <c r="I10" s="111"/>
-      <c r="J10" s="112"/>
-      <c r="K10" s="113" t="s">
-        <v>225</v>
-      </c>
-      <c r="L10" s="114"/>
-      <c r="M10" s="114"/>
-      <c r="N10" s="115"/>
-      <c r="O10" s="133" t="s">
-        <v>222</v>
-      </c>
-      <c r="P10" s="133"/>
-      <c r="Q10" s="134"/>
-      <c r="R10" s="135" t="s">
-        <v>223</v>
-      </c>
-      <c r="S10" s="136"/>
-      <c r="T10" s="136"/>
-      <c r="U10" s="136"/>
-      <c r="V10" s="137"/>
-      <c r="W10" s="138" t="s">
-        <v>226</v>
-      </c>
-      <c r="X10" s="139"/>
-      <c r="Y10" s="139"/>
-      <c r="Z10" s="140"/>
+      <c r="S10" s="124"/>
+      <c r="T10" s="124"/>
+      <c r="U10" s="124"/>
+      <c r="V10" s="125"/>
+      <c r="W10" s="120" t="s">
+        <v>224</v>
+      </c>
+      <c r="X10" s="121"/>
+      <c r="Y10" s="121"/>
+      <c r="Z10" s="122"/>
       <c r="AB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="116" t="s">
+      <c r="AC10" s="127" t="s">
+        <v>225</v>
+      </c>
+      <c r="AD10" s="127"/>
+      <c r="AE10" s="128"/>
+      <c r="AF10" s="129" t="s">
+        <v>226</v>
+      </c>
+      <c r="AG10" s="130"/>
+      <c r="AH10" s="130"/>
+      <c r="AI10" s="130"/>
+      <c r="AJ10" s="131"/>
+      <c r="AK10" s="132" t="s">
         <v>227</v>
       </c>
-      <c r="AD10" s="116"/>
-      <c r="AE10" s="117"/>
-      <c r="AF10" s="118" t="s">
+      <c r="AL10" s="133"/>
+      <c r="AM10" s="133"/>
+      <c r="AN10" s="134"/>
+      <c r="AO10" s="135" t="s">
         <v>228</v>
       </c>
-      <c r="AG10" s="119"/>
-      <c r="AH10" s="119"/>
-      <c r="AI10" s="119"/>
-      <c r="AJ10" s="120"/>
-      <c r="AK10" s="121" t="s">
+      <c r="AP10" s="136"/>
+      <c r="AQ10" s="137"/>
+      <c r="AR10" s="138" t="s">
         <v>229</v>
       </c>
-      <c r="AL10" s="122"/>
-      <c r="AM10" s="122"/>
-      <c r="AN10" s="123"/>
-      <c r="AO10" s="124" t="s">
+      <c r="AS10" s="139"/>
+      <c r="AT10" s="139"/>
+      <c r="AU10" s="139"/>
+      <c r="AV10" s="140"/>
+      <c r="AW10" s="114" t="s">
         <v>230</v>
       </c>
-      <c r="AP10" s="125"/>
-      <c r="AQ10" s="126"/>
-      <c r="AR10" s="127" t="s">
-        <v>231</v>
-      </c>
-      <c r="AS10" s="128"/>
-      <c r="AT10" s="128"/>
-      <c r="AU10" s="128"/>
-      <c r="AV10" s="129"/>
-      <c r="AW10" s="130" t="s">
-        <v>232</v>
-      </c>
-      <c r="AX10" s="131"/>
-      <c r="AY10" s="131"/>
-      <c r="AZ10" s="132"/>
+      <c r="AX10" s="115"/>
+      <c r="AY10" s="115"/>
+      <c r="AZ10" s="116"/>
       <c r="BB10" s="45" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="108" t="s">
+      <c r="BC10" s="107" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD10" s="107"/>
+      <c r="BE10" s="108"/>
+      <c r="BF10" s="111" t="s">
+        <v>232</v>
+      </c>
+      <c r="BG10" s="112"/>
+      <c r="BH10" s="112"/>
+      <c r="BI10" s="112"/>
+      <c r="BJ10" s="113"/>
+      <c r="BK10" s="117" t="s">
         <v>233</v>
       </c>
-      <c r="BD10" s="108"/>
-      <c r="BE10" s="109"/>
-      <c r="BF10" s="110" t="s">
+      <c r="BL10" s="118"/>
+      <c r="BM10" s="118"/>
+      <c r="BN10" s="119"/>
+      <c r="BO10" s="109" t="s">
+        <v>239</v>
+      </c>
+      <c r="BP10" s="109"/>
+      <c r="BQ10" s="110"/>
+      <c r="BR10" s="123" t="s">
+        <v>240</v>
+      </c>
+      <c r="BS10" s="124"/>
+      <c r="BT10" s="124"/>
+      <c r="BU10" s="124"/>
+      <c r="BV10" s="125"/>
+      <c r="BW10" s="120" t="s">
         <v>234</v>
       </c>
-      <c r="BG10" s="111"/>
-      <c r="BH10" s="111"/>
-      <c r="BI10" s="111"/>
-      <c r="BJ10" s="112"/>
-      <c r="BK10" s="113" t="s">
-        <v>235</v>
-      </c>
-      <c r="BL10" s="114"/>
-      <c r="BM10" s="114"/>
-      <c r="BN10" s="115"/>
-      <c r="BO10" s="133" t="s">
-        <v>241</v>
-      </c>
-      <c r="BP10" s="133"/>
-      <c r="BQ10" s="134"/>
-      <c r="BR10" s="135" t="s">
-        <v>242</v>
-      </c>
-      <c r="BS10" s="136"/>
-      <c r="BT10" s="136"/>
-      <c r="BU10" s="136"/>
-      <c r="BV10" s="137"/>
-      <c r="BW10" s="138" t="s">
-        <v>236</v>
-      </c>
-      <c r="BX10" s="139"/>
-      <c r="BY10" s="139"/>
-      <c r="BZ10" s="140"/>
+      <c r="BX10" s="121"/>
+      <c r="BY10" s="121"/>
+      <c r="BZ10" s="122"/>
     </row>
-    <row r="11" spans="1:78" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="107"/>
+    <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A11" s="126"/>
       <c r="B11" s="46" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C11" s="58" t="str">
         <f ca="1">CONCATENATE("≤",YEAR(TODAY())-15)</f>
@@ -18080,7 +18080,7 @@
       </c>
       <c r="AA11" s="39"/>
       <c r="AB11" s="46" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="AC11" s="80" t="str">
         <f ca="1">CONCATENATE("≤",YEAR(TODAY())-15)</f>
@@ -18179,7 +18179,7 @@
         <v>2002-1986</v>
       </c>
       <c r="BB11" s="46" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="BC11" s="58" t="str">
         <f ca="1">CONCATENATE("≤",YEAR(TODAY())-15-1)</f>
@@ -18278,8 +18278,8 @@
         <v>2001-1985</v>
       </c>
     </row>
-    <row r="12" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="107"/>
+    <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="126"/>
       <c r="B12" s="47" t="s">
         <v>0</v>
       </c>
@@ -18530,8 +18530,8 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A13" s="107"/>
+    <row r="13" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A13" s="126"/>
       <c r="B13" s="47" t="s">
         <v>185</v>
       </c>
@@ -18782,8 +18782,8 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A14" s="107"/>
+    <row r="14" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A14" s="126"/>
       <c r="B14" s="47" t="s">
         <v>186</v>
       </c>
@@ -19034,8 +19034,8 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A15" s="107"/>
+    <row r="15" spans="1:78" x14ac:dyDescent="0.45">
+      <c r="A15" s="126"/>
       <c r="B15" s="47" t="s">
         <v>187</v>
       </c>
@@ -19286,8 +19286,8 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="107"/>
+    <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="126"/>
       <c r="B16" s="47" t="s">
         <v>188</v>
       </c>
@@ -19538,8 +19538,8 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:78" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="107"/>
+    <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A17" s="126"/>
       <c r="B17" s="50" t="s">
         <v>4</v>
       </c>
@@ -19790,7 +19790,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:78" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="C18" s="30"/>
       <c r="O18" s="30"/>
       <c r="T18" s="33"/>
@@ -19799,7 +19799,7 @@
       <c r="X18" s="30"/>
       <c r="AD18" s="30"/>
     </row>
-    <row r="21" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C21" s="29"/>
       <c r="D21" s="32"/>
       <c r="E21" s="32"/>
@@ -19819,7 +19819,7 @@
       <c r="AF21" s="35"/>
       <c r="AG21" s="35"/>
     </row>
-    <row r="22" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C22" s="30"/>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -19839,7 +19839,7 @@
       <c r="AF22" s="31"/>
       <c r="AG22" s="31"/>
     </row>
-    <row r="23" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C23" s="30"/>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -19859,7 +19859,7 @@
       <c r="AF23" s="31"/>
       <c r="AG23" s="31"/>
     </row>
-    <row r="24" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C24" s="30"/>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -19879,7 +19879,7 @@
       <c r="AF24" s="31"/>
       <c r="AG24" s="31"/>
     </row>
-    <row r="25" spans="1:78" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:78" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C25" s="30"/>
       <c r="D25" s="31"/>
       <c r="E25" s="31"/>
@@ -19899,7 +19899,7 @@
       <c r="AF25" s="31"/>
       <c r="AG25" s="31"/>
     </row>
-    <row r="26" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C26" s="30"/>
       <c r="D26" s="31"/>
       <c r="E26" s="31"/>
@@ -19919,7 +19919,7 @@
       <c r="AF26" s="31"/>
       <c r="AG26" s="31"/>
     </row>
-    <row r="27" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C27" s="30"/>
       <c r="D27" s="31"/>
       <c r="E27" s="31"/>
@@ -19939,7 +19939,7 @@
       <c r="AF27" s="31"/>
       <c r="AG27" s="31"/>
     </row>
-    <row r="30" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C30" s="29"/>
       <c r="D30" s="32"/>
       <c r="E30" s="32"/>
@@ -19948,7 +19948,7 @@
       <c r="H30" s="32"/>
       <c r="P30" s="33"/>
     </row>
-    <row r="31" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:78" x14ac:dyDescent="0.45">
       <c r="C31" s="30"/>
       <c r="D31" s="31"/>
       <c r="E31" s="31"/>
@@ -19956,7 +19956,7 @@
       <c r="G31" s="31"/>
       <c r="H31" s="31"/>
     </row>
-    <row r="40" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C40" s="30"/>
       <c r="D40" s="31"/>
       <c r="E40" s="31"/>
@@ -19964,7 +19964,7 @@
       <c r="G40" s="31"/>
       <c r="H40" s="31"/>
     </row>
-    <row r="41" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C41" s="30"/>
       <c r="D41" s="31"/>
       <c r="E41" s="31"/>
@@ -19972,7 +19972,7 @@
       <c r="G41" s="31"/>
       <c r="H41" s="31"/>
     </row>
-    <row r="42" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C42" s="30"/>
       <c r="D42" s="31"/>
       <c r="E42" s="31"/>
@@ -19980,7 +19980,7 @@
       <c r="G42" s="31"/>
       <c r="H42" s="31"/>
     </row>
-    <row r="43" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C43" s="30"/>
       <c r="D43" s="31"/>
       <c r="E43" s="31"/>
@@ -19988,7 +19988,7 @@
       <c r="G43" s="31"/>
       <c r="H43" s="31"/>
     </row>
-    <row r="44" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C44" s="30"/>
       <c r="D44" s="31"/>
       <c r="E44" s="31"/>
@@ -19996,7 +19996,7 @@
       <c r="G44" s="31"/>
       <c r="H44" s="31"/>
     </row>
-    <row r="45" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C45" s="30"/>
       <c r="D45" s="31"/>
       <c r="E45" s="31"/>
@@ -20006,28 +20006,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -20044,6 +20022,28 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">

</xml_diff>

<commit_message>
WR Korrektur & DEM Tag 3 Complete
</commit_message>
<xml_diff>
--- a/web/data/records_kriterien.xlsx
+++ b/web/data/records_kriterien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C295E636-7E52-4533-AA3C-CE7221D5C361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DB0669-4FB4-4BAB-93C2-8FE76442A827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" activeTab="2" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
@@ -1706,16 +1706,17 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1727,15 +1728,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1744,27 +1736,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1808,8 +1779,37 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1817,7 +1817,7 @@
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="259">
+  <dxfs count="261">
     <dxf>
       <font>
         <color theme="4"/>
@@ -1825,7 +1825,32 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0" tint="-0.24994659260841701"/>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="4"/>
       </font>
     </dxf>
     <dxf>
@@ -1835,7 +1860,7 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="6"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </font>
     </dxf>
     <dxf>
@@ -1845,7 +1870,7 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="4"/>
+        <color theme="6"/>
       </font>
     </dxf>
     <dxf>
@@ -1855,7 +1880,7 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="6"/>
+        <color theme="4"/>
       </font>
     </dxf>
     <dxf>
@@ -1870,6 +1895,11 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="4"/>
       </font>
     </dxf>
@@ -1904,26 +1934,6 @@
       </font>
     </dxf>
     <dxf>
-      <font>
-        <color theme="6"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="6"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="4"/>
-      </font>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2156,39 +2166,51 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2207,12 +2229,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2222,6 +2247,84 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2360,6 +2463,110 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2613,6 +2820,31 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="medium">
           <color theme="0"/>
@@ -2669,6 +2901,349 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <vertical/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -2968,431 +3543,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="medium">
-          <color theme="3" tint="-0.499984740745262"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <vertical/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <vertical/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -3721,30 +3871,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="medium">
@@ -3752,84 +3878,6 @@
         </right>
         <vertical/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -4050,13 +4098,68 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <right style="medium">
-          <color indexed="64"/>
+          <color theme="3" tint="-0.499984740745262"/>
         </right>
-        <vertical/>
       </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -4338,100 +4441,7 @@
           <bgColor theme="6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4447,60 +4457,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="232" headerRowBorderDxfId="231" tableBorderDxfId="230">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="248" headerRowBorderDxfId="247" tableBorderDxfId="246">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="229">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="245">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="228"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="227"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="226"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="225"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="224"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="223"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="222"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="221"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="244"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="243"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="242"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="241"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="240"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="239"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="238"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="237"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="220"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="219"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="218"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="217"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="216"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="215"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="214"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="213"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="212"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="211"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="210"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="209"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="208"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="207"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="206"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="205"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="204"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="203"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="202"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="201"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="200"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="199"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="198"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="197"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="196"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="195"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="194"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="193"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="192"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="191"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="190"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="189"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="188"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="187"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="186"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="185"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="184"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="236"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="235"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="234"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="233"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="232"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="231"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="230"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="229"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="228"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="227"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="226"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="225"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="224"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="223"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="222"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="221"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="220"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="219"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="218"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="217"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="216"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="215"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="214"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="213"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="212"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="211"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="210"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="209"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="208"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="207"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="206"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="205"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="204"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="203"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="202"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="201"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="200"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4510,12 +4520,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}" name="LK_Kalender" displayName="LK_Kalender" ref="A1:H14" totalsRowShown="0">
   <autoFilter ref="A1:H14" xr:uid="{888CE7BE-8313-44C0-AE38-83992EABD44D}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{B26B9E90-F378-41EF-B35E-CE240017E4BE}" name="datum von" dataDxfId="27"/>
     <tableColumn id="2" xr3:uid="{38211212-0A92-428C-895C-E4CA68F52818}" name="datum bis"/>
-    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{66E541C6-0A5E-4B2D-9B89-5E52F449A4A6}" name="uhrzeit von" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{D93C06A2-29AD-4073-8E3C-A685B4474CC8}" name="uhrzeit bis" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{C5C3979C-B528-44E8-A5A6-36F020A6034F}" name="titel" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{9DC09E1D-44FD-40ED-9EBE-86A8E61C38B2}" name="meta" dataDxfId="23"/>
     <tableColumn id="7" xr3:uid="{E7E62A34-7A76-4361-937D-F4DE76E6E7CC}" name="ort"/>
     <tableColumn id="8" xr3:uid="{84F02734-FC16-406B-ACCA-0CCDF547D94C}" name="kader"/>
   </tableColumns>
@@ -4524,42 +4534,42 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="183" dataDxfId="181" headerRowBorderDxfId="182" tableBorderDxfId="180">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="199" dataDxfId="197" headerRowBorderDxfId="198" tableBorderDxfId="196">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="179"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="178"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="177"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="176"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="175"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="174"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="173"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="172"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="171"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="170"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="169"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="168"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="167"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="195"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="194"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="193"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="192"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="191"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="190"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="189"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="188"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="187"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="186"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="185"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="184"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="183"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="166" headerRowBorderDxfId="165" tableBorderDxfId="164">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="260" headerRowBorderDxfId="259" tableBorderDxfId="258">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="163">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="257">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="162"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="161"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="160"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="159"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="158"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="157"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="156"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="155"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="256"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="255"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="254"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="253"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="252"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="251"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="250"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="249"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -4570,7 +4580,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="154" dataDxfId="153">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}" name="DP_konfig" displayName="DP_konfig" ref="A1:U3" totalsRowShown="0" headerRowDxfId="182" dataDxfId="181">
   <autoFilter ref="A1:U3" xr:uid="{CF3D303A-A04B-42DD-A44E-CEB6CECB77A4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4595,94 +4605,94 @@
     <filterColumn colId="20" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="152"/>
-    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="151"/>
-    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="150"/>
-    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="149"/>
-    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="148"/>
-    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="147"/>
-    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="146"/>
-    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="145"/>
-    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="144"/>
-    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="143"/>
-    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="142"/>
-    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="141"/>
-    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="140"/>
-    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="139"/>
-    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="138"/>
-    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="137"/>
-    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="136"/>
-    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="135"/>
-    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="134"/>
-    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="133"/>
-    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="132"/>
+    <tableColumn id="1" xr3:uid="{58D628F0-061E-4A82-8362-CDB37A2E7C60}" name="Tabellen Name" dataDxfId="180"/>
+    <tableColumn id="2" xr3:uid="{2F302F6C-F8AF-4FDE-AB08-6F30F9671015}" name="Geschlecht" dataDxfId="179"/>
+    <tableColumn id="3" xr3:uid="{4D91FBF9-386D-43DD-90D0-B49823FDB629}" name="Mindest alter" dataDxfId="178"/>
+    <tableColumn id="4" xr3:uid="{4126AAC6-AF2F-446C-B4EA-D86ACFD9FAC2}" name="Maximales Alter" dataDxfId="177"/>
+    <tableColumn id="5" xr3:uid="{8A10890A-A299-4B09-AC72-0E9AE9238AF3}" name="Qualizeitraum anfang" dataDxfId="176"/>
+    <tableColumn id="6" xr3:uid="{FBCD1C13-FC82-429B-8DE1-0C5A455FDAB8}" name="Qualizeitraum Ende" dataDxfId="175"/>
+    <tableColumn id="7" xr3:uid="{1DCCAC9B-BC46-468E-A3CE-57576C2FF11D}" name="Letzter Wettkampf am" dataDxfId="174"/>
+    <tableColumn id="8" xr3:uid="{9A6E47EE-ABD8-4A1E-87D3-9D286E4C124F}" name="Wertung" dataDxfId="173"/>
+    <tableColumn id="9" xr3:uid="{09E848D2-ED17-49C7-9775-CBF17D20DFC0}" name="Landesverband" dataDxfId="172"/>
+    <tableColumn id="10" xr3:uid="{70ABB713-23F6-4FCF-920E-3CB0CD451446}" name="OMS" dataDxfId="171"/>
+    <tableColumn id="11" xr3:uid="{9C108A1C-E6AB-4C13-9C1D-0FA8944A39A3}" name="Pool-Länge" dataDxfId="170"/>
+    <tableColumn id="12" xr3:uid="{087948DD-430D-48F1-906D-4F4EF4B46053}" name="Regelwerk" dataDxfId="169"/>
+    <tableColumn id="13" xr3:uid="{BF42D9C0-F77D-4971-A67E-32B0246C72C3}" name="Referenz" dataDxfId="168"/>
+    <tableColumn id="19" xr3:uid="{AFFB84E8-B398-4E99-805B-9A247071A040}" name="Referenz Jahr" dataDxfId="167"/>
+    <tableColumn id="20" xr3:uid="{0A59A474-DFBB-4437-8EFF-70284AFD9934}" name="Mindest Punktzahl" dataDxfId="166"/>
+    <tableColumn id="21" xr3:uid="{198BD231-EEF3-43C9-AD9B-39B4B7E9B337}" name="Mindest Disziplinen" dataDxfId="165"/>
+    <tableColumn id="14" xr3:uid="{443CD4F6-A2B2-480B-BB35-DCEEBC531727}" name="3-Kampf Regel" dataDxfId="164"/>
+    <tableColumn id="15" xr3:uid="{70116160-7666-42B1-92AC-FAC2620E6A60}" name="Anzahl Nominierte" dataDxfId="163"/>
+    <tableColumn id="16" xr3:uid="{0EFD0A46-D12B-4AB0-907C-08E5D9F282E0}" name="Anzahl Nachrücker" dataDxfId="162"/>
+    <tableColumn id="17" xr3:uid="{AA5430A0-8ED8-40E8-B7F8-DA25E4E8790F}" name="Seiten Anzahl" dataDxfId="161"/>
+    <tableColumn id="18" xr3:uid="{16F699D9-2741-43F3-AD5F-826A568EFEAC}" name="Absagen" dataDxfId="160"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="131" dataDxfId="130">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}" name="BP_konfig" displayName="BP_konfig" ref="A1:U7" totalsRowShown="0" headerRowDxfId="159" dataDxfId="158">
   <autoFilter ref="A1:U7" xr:uid="{CDBF6724-48A1-41AB-94B5-CC35C54BB15C}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="129"/>
-    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="128"/>
-    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="127"/>
-    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="126"/>
-    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="125"/>
-    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="124"/>
-    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="123"/>
-    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="122"/>
-    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="121"/>
-    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="120"/>
-    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="119"/>
-    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="118"/>
-    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="117"/>
-    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="116"/>
-    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="115"/>
-    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="114"/>
-    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="113"/>
-    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="112"/>
-    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="111"/>
-    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="110"/>
-    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="109"/>
+    <tableColumn id="1" xr3:uid="{E1FB3D0C-B874-4874-BACC-6872CF171957}" name="Tabellen Name" dataDxfId="157"/>
+    <tableColumn id="2" xr3:uid="{FFDD2777-2097-450C-B020-F133CF643855}" name="Geschlecht" dataDxfId="156"/>
+    <tableColumn id="3" xr3:uid="{8CF52BE2-8020-48BD-A36D-63F13A1878DE}" name="Mindest alter" dataDxfId="155"/>
+    <tableColumn id="4" xr3:uid="{FD3A030F-CD97-4B6F-8E8C-BC2E67D79F1D}" name="Maximales Alter" dataDxfId="154"/>
+    <tableColumn id="5" xr3:uid="{3E22B645-D77C-4509-B031-9914FCB91599}" name="Qualizeitraum anfang" dataDxfId="153"/>
+    <tableColumn id="6" xr3:uid="{AE299324-3C1C-4063-ADF9-54555A161734}" name="Qualizeitraum Ende" dataDxfId="152"/>
+    <tableColumn id="7" xr3:uid="{DCC178B3-11FC-4C53-BBC6-C2FDA2C89857}" name="Letzter Wettkampf am" dataDxfId="151"/>
+    <tableColumn id="8" xr3:uid="{2811DB01-60A5-4BE4-B6F9-A806398A602A}" name="Wertung" dataDxfId="150"/>
+    <tableColumn id="9" xr3:uid="{0C16DAFE-847D-4E9E-9604-3A7D9FE924D0}" name="Landesverband" dataDxfId="149"/>
+    <tableColumn id="10" xr3:uid="{7A8A4101-A553-4BD5-9116-9AA5876B9401}" name="OMS" dataDxfId="148"/>
+    <tableColumn id="11" xr3:uid="{9807C9BD-6499-45F6-ACE0-4D13D64EF675}" name="Pool-Länge" dataDxfId="147"/>
+    <tableColumn id="12" xr3:uid="{13D336DD-650F-4F2C-836F-361CA1528F6D}" name="Regelwerk" dataDxfId="146"/>
+    <tableColumn id="13" xr3:uid="{66660E2D-ADF2-4FB5-8A13-004F826EE908}" name="Referenz" dataDxfId="145"/>
+    <tableColumn id="19" xr3:uid="{D72EDF8B-ECC3-4FF7-ABE6-B60BCE4A5E26}" name="Referenz Jahr" dataDxfId="144"/>
+    <tableColumn id="20" xr3:uid="{7B18E667-70F7-4BC1-AB1B-21C019F2AA89}" name="Mindest Punktzahl" dataDxfId="143"/>
+    <tableColumn id="21" xr3:uid="{FC185946-681B-42A6-AB1A-FC1EABB668C5}" name="Mindest Disziplinen" dataDxfId="142"/>
+    <tableColumn id="14" xr3:uid="{6A2676FD-2EC7-4C41-A35E-A1597A38F932}" name="3-Kampf Regel" dataDxfId="141"/>
+    <tableColumn id="15" xr3:uid="{718E0917-4F83-4A2B-832F-EBB16D5E21BF}" name="Anzahl Nominierte" dataDxfId="140"/>
+    <tableColumn id="16" xr3:uid="{5C66A461-D647-4E00-A81C-FD7AD44D7CC2}" name="Anzahl Nachrücker" dataDxfId="139"/>
+    <tableColumn id="17" xr3:uid="{D434BDEC-293B-4B4E-A5E9-479438960A03}" name="Seiten Anzahl" dataDxfId="138"/>
+    <tableColumn id="18" xr3:uid="{80908229-9247-473F-81C0-9C9D4C12FF06}" name="Absagen" dataDxfId="137"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9BFD34D3-012E-42D2-B8D4-32612CAE2B03}" name="Natio_konfig" displayName="Natio_konfig" ref="A1:U5" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9BFD34D3-012E-42D2-B8D4-32612CAE2B03}" name="Natio_konfig" displayName="Natio_konfig" ref="A1:U5" totalsRowShown="0" headerRowDxfId="136" dataDxfId="135">
   <autoFilter ref="A1:U5" xr:uid="{9BFD34D3-012E-42D2-B8D4-32612CAE2B03}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{5F38FA64-1E26-48F3-B0FF-0E5583AED772}" name="Tabellen Name" dataDxfId="106"/>
-    <tableColumn id="2" xr3:uid="{5F8CE91B-BB92-40A2-8EC5-CAA4A0736BC7}" name="Geschlecht" dataDxfId="105"/>
-    <tableColumn id="3" xr3:uid="{BABC4117-3513-4A51-88FC-ACCDE4FEA695}" name="Mindest alter" dataDxfId="104"/>
-    <tableColumn id="4" xr3:uid="{CCAD214E-6485-4A99-9B76-61FD1F836615}" name="Maximales Alter" dataDxfId="103"/>
-    <tableColumn id="5" xr3:uid="{D40FDC2D-1060-4B9A-9D8D-DE371966BAAB}" name="Qualizeitraum anfang" dataDxfId="102"/>
-    <tableColumn id="6" xr3:uid="{2FB5B18D-9671-410E-820E-4F8AAAB94AE5}" name="Qualizeitraum Ende" dataDxfId="101"/>
-    <tableColumn id="7" xr3:uid="{78B05291-7E65-403E-9E77-08F9F175C88E}" name="Letzter Wettkampf am" dataDxfId="100"/>
-    <tableColumn id="8" xr3:uid="{E0DF794B-64F4-4803-A055-5B5D5AC5C173}" name="Wertung" dataDxfId="99"/>
-    <tableColumn id="9" xr3:uid="{7DC0795F-A548-4A09-8FFF-04A3E561E613}" name="Landesverband" dataDxfId="98"/>
-    <tableColumn id="10" xr3:uid="{FBA31A17-CE11-420F-9487-0A4D973C90F9}" name="OMS" dataDxfId="97"/>
-    <tableColumn id="11" xr3:uid="{60B8D281-E504-4B42-81B8-9B14A1A926A0}" name="Pool-Länge" dataDxfId="96"/>
-    <tableColumn id="12" xr3:uid="{E4E00861-E0C2-470C-ACC3-AEB71183E69E}" name="Regelwerk" dataDxfId="95"/>
-    <tableColumn id="13" xr3:uid="{67DAD4F5-E83D-48A3-9BA2-9B3F5710FEC3}" name="Referenz" dataDxfId="94"/>
-    <tableColumn id="19" xr3:uid="{DCD9D3BE-5C04-4575-92EC-F8E911242805}" name="Referenz Jahr" dataDxfId="93"/>
-    <tableColumn id="20" xr3:uid="{3B307C90-C4F5-4890-BF5F-3499E6C4E068}" name="Mindest Punktzahl" dataDxfId="92"/>
-    <tableColumn id="21" xr3:uid="{759A1906-0454-4CC4-8BED-31ABBD324EC9}" name="Mindest Disziplinen" dataDxfId="91"/>
-    <tableColumn id="14" xr3:uid="{41BD1BD0-16DC-4E03-AF06-BE8444616C3A}" name="3-Kampf Regel" dataDxfId="90"/>
-    <tableColumn id="15" xr3:uid="{FCA10EFA-53B1-4722-9BA3-416DC54A7205}" name="Anzahl Nominierte" dataDxfId="89"/>
-    <tableColumn id="16" xr3:uid="{A17696BB-052A-4E5D-916A-75001AA350CB}" name="Anzahl Nachrücker" dataDxfId="88"/>
-    <tableColumn id="17" xr3:uid="{7DC8C503-FEE5-46A4-B2AB-C5627D45C70D}" name="Seiten Anzahl" dataDxfId="87"/>
-    <tableColumn id="18" xr3:uid="{5F4E44AE-8D26-45E0-A15C-6CA7D8FA4819}" name="Absagen" dataDxfId="86"/>
+    <tableColumn id="1" xr3:uid="{5F38FA64-1E26-48F3-B0FF-0E5583AED772}" name="Tabellen Name" dataDxfId="134"/>
+    <tableColumn id="2" xr3:uid="{5F8CE91B-BB92-40A2-8EC5-CAA4A0736BC7}" name="Geschlecht" dataDxfId="133"/>
+    <tableColumn id="3" xr3:uid="{BABC4117-3513-4A51-88FC-ACCDE4FEA695}" name="Mindest alter" dataDxfId="132"/>
+    <tableColumn id="4" xr3:uid="{CCAD214E-6485-4A99-9B76-61FD1F836615}" name="Maximales Alter" dataDxfId="131"/>
+    <tableColumn id="5" xr3:uid="{D40FDC2D-1060-4B9A-9D8D-DE371966BAAB}" name="Qualizeitraum anfang" dataDxfId="130"/>
+    <tableColumn id="6" xr3:uid="{2FB5B18D-9671-410E-820E-4F8AAAB94AE5}" name="Qualizeitraum Ende" dataDxfId="129"/>
+    <tableColumn id="7" xr3:uid="{78B05291-7E65-403E-9E77-08F9F175C88E}" name="Letzter Wettkampf am" dataDxfId="128"/>
+    <tableColumn id="8" xr3:uid="{E0DF794B-64F4-4803-A055-5B5D5AC5C173}" name="Wertung" dataDxfId="127"/>
+    <tableColumn id="9" xr3:uid="{7DC0795F-A548-4A09-8FFF-04A3E561E613}" name="Landesverband" dataDxfId="126"/>
+    <tableColumn id="10" xr3:uid="{FBA31A17-CE11-420F-9487-0A4D973C90F9}" name="OMS" dataDxfId="125"/>
+    <tableColumn id="11" xr3:uid="{60B8D281-E504-4B42-81B8-9B14A1A926A0}" name="Pool-Länge" dataDxfId="124"/>
+    <tableColumn id="12" xr3:uid="{E4E00861-E0C2-470C-ACC3-AEB71183E69E}" name="Regelwerk" dataDxfId="123"/>
+    <tableColumn id="13" xr3:uid="{67DAD4F5-E83D-48A3-9BA2-9B3F5710FEC3}" name="Referenz" dataDxfId="122"/>
+    <tableColumn id="19" xr3:uid="{DCD9D3BE-5C04-4575-92EC-F8E911242805}" name="Referenz Jahr" dataDxfId="121"/>
+    <tableColumn id="20" xr3:uid="{3B307C90-C4F5-4890-BF5F-3499E6C4E068}" name="Mindest Punktzahl" dataDxfId="120"/>
+    <tableColumn id="21" xr3:uid="{759A1906-0454-4CC4-8BED-31ABBD324EC9}" name="Mindest Disziplinen" dataDxfId="119"/>
+    <tableColumn id="14" xr3:uid="{41BD1BD0-16DC-4E03-AF06-BE8444616C3A}" name="3-Kampf Regel" dataDxfId="118"/>
+    <tableColumn id="15" xr3:uid="{FCA10EFA-53B1-4722-9BA3-416DC54A7205}" name="Anzahl Nominierte" dataDxfId="117"/>
+    <tableColumn id="16" xr3:uid="{A17696BB-052A-4E5D-916A-75001AA350CB}" name="Anzahl Nachrücker" dataDxfId="116"/>
+    <tableColumn id="17" xr3:uid="{7DC8C503-FEE5-46A4-B2AB-C5627D45C70D}" name="Seiten Anzahl" dataDxfId="115"/>
+    <tableColumn id="18" xr3:uid="{5F4E44AE-8D26-45E0-A15C-6CA7D8FA4819}" name="Absagen" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}" name="DEM_konfig" displayName="DEM_konfig" ref="A1:X7" totalsRowShown="0" headerRowDxfId="113" dataDxfId="112">
   <autoFilter ref="A1:X7" xr:uid="{16F87202-5A6A-4E2F-B973-3CE7EC2566C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4710,37 +4720,37 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="83"/>
-    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="82"/>
-    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="80"/>
-    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="79"/>
-    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="78"/>
-    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="77"/>
-    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="75"/>
-    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="74"/>
-    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="73"/>
-    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="72"/>
-    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="71"/>
-    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="70"/>
-    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="69"/>
-    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="68"/>
-    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="67"/>
-    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="66"/>
-    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="65"/>
-    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="64"/>
-    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="63"/>
-    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="62"/>
-    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="61"/>
-    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{4847B567-64E1-4AC3-8C4B-EFCF3F00CC6C}" name="Tabellen Name" dataDxfId="111"/>
+    <tableColumn id="2" xr3:uid="{6346FF3B-B334-4CD8-8B23-F2347E29C536}" name="Geschlecht" dataDxfId="110"/>
+    <tableColumn id="3" xr3:uid="{E793B48A-BC8A-439F-8AAF-6FD08104A619}" name="Mindest Alter" dataDxfId="109"/>
+    <tableColumn id="4" xr3:uid="{01A62C29-2F75-4107-A431-F69230BCCD0C}" name="Maximales Alter" dataDxfId="108"/>
+    <tableColumn id="5" xr3:uid="{B7E4DE90-7856-4A0C-9063-61414D7F227C}" name="Qualizeitraum anfang" dataDxfId="107"/>
+    <tableColumn id="6" xr3:uid="{B00F7CD1-82CB-42B9-A396-89F79EF419CA}" name="Qualizeitraum Ende" dataDxfId="106"/>
+    <tableColumn id="7" xr3:uid="{9E50DDE5-12E3-4BCB-801C-FBABCE309F0E}" name="Letzter Wettkampf am" dataDxfId="105"/>
+    <tableColumn id="8" xr3:uid="{57E68247-0FF2-48D8-8ACD-AB057E576A21}" name="Landesverband" dataDxfId="104"/>
+    <tableColumn id="9" xr3:uid="{EBAA439D-F69A-4C2A-8193-9AE08F1E57B8}" name="OMS" dataDxfId="103"/>
+    <tableColumn id="10" xr3:uid="{BBD11E7F-3DDF-428A-B005-4A40E6FA78DC}" name="Pool-Länge" dataDxfId="102"/>
+    <tableColumn id="11" xr3:uid="{6AE38DCA-A084-4F3D-A6A4-4E76E3E2CBC6}" name="Regelwerk" dataDxfId="101"/>
+    <tableColumn id="12" xr3:uid="{7F7470AD-5502-4CEE-BB4C-44BA308E61D7}" name="Seiten Anzahl" dataDxfId="100"/>
+    <tableColumn id="13" xr3:uid="{F416CBFA-4C9D-45CD-9BA7-E4BC57A08BC2}" name="PZ1 - 50m Retten" dataDxfId="99"/>
+    <tableColumn id="14" xr3:uid="{7117DBCA-0DA7-462C-84FE-0DC7E33B124C}" name="PZ1 - 100m Retten" dataDxfId="98"/>
+    <tableColumn id="15" xr3:uid="{E8630E91-DC30-4822-9E53-6D65487C3670}" name="PZ1 - 100m Kombi" dataDxfId="97"/>
+    <tableColumn id="16" xr3:uid="{4B3AA225-E042-430F-8259-D176887B4528}" name="PZ1 - 100m Lifesaver" dataDxfId="96"/>
+    <tableColumn id="17" xr3:uid="{798674BD-98CE-4531-BDFF-6AB06253AD7C}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="95"/>
+    <tableColumn id="18" xr3:uid="{8809BB71-D58B-4E8B-A442-D0EB9A65A25D}" name="PZ1 - 200m Hindernis" dataDxfId="94"/>
+    <tableColumn id="19" xr3:uid="{93DCF463-806B-4117-B4E3-1FFAE976B37C}" name="PZ2 - 50m Retten" dataDxfId="93"/>
+    <tableColumn id="20" xr3:uid="{A514C961-559E-462F-B143-BA30974C0129}" name="PZ2 - 100m Retten" dataDxfId="92"/>
+    <tableColumn id="21" xr3:uid="{F1CF6143-45FE-498D-93D6-36F26D2F3C0B}" name="PZ2 - 100m Kombi" dataDxfId="91"/>
+    <tableColumn id="22" xr3:uid="{E90962FC-C214-467F-841F-40DF60E41456}" name="PZ2 - 100m Lifesaver" dataDxfId="90"/>
+    <tableColumn id="23" xr3:uid="{7FBC6334-C4C8-4B38-9F59-30ED95A44379}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="89"/>
+    <tableColumn id="24" xr3:uid="{231BFF86-8F3A-4BA1-B25E-28175D9EDFA9}" name="PZ2 - 200m Hindernis" dataDxfId="88"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="258" dataDxfId="257">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}" name="JRP_konfig" displayName="JRP_konfig" ref="A1:X3" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
   <autoFilter ref="A1:X3" xr:uid="{D7CDEF11-F813-469D-9DE0-678961AB7005}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4768,71 +4778,71 @@
     <filterColumn colId="23" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="256"/>
-    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="255"/>
-    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="254"/>
-    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="253"/>
-    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="252"/>
-    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="251"/>
-    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="250"/>
-    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="249"/>
-    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="248"/>
-    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="247"/>
-    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="246"/>
-    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="245"/>
-    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="244"/>
-    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="243"/>
-    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="242"/>
-    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="241"/>
-    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="240"/>
-    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="239"/>
-    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="238"/>
-    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="237"/>
-    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="236"/>
-    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="235"/>
-    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="234"/>
-    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="233"/>
+    <tableColumn id="1" xr3:uid="{021DA6E1-2C93-4474-9720-B6F016186D61}" name="Tabellen Name" dataDxfId="85"/>
+    <tableColumn id="2" xr3:uid="{733C1722-A9C9-4830-A9E2-FE62E96BCD98}" name="Geschlecht" dataDxfId="84"/>
+    <tableColumn id="3" xr3:uid="{80C0BF46-0E43-4947-BF86-B808C324772A}" name="Mindest Alter" dataDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{DBA2A923-EEB7-43F9-A1A3-E78624448FB9}" name="Maximales Alter" dataDxfId="82"/>
+    <tableColumn id="5" xr3:uid="{3FDEE18A-328D-45AE-907D-69A916A93345}" name="Qualizeitraum anfang" dataDxfId="81"/>
+    <tableColumn id="6" xr3:uid="{BE002D7F-575F-4B60-9251-C71D93F59045}" name="Qualizeitraum Ende" dataDxfId="80"/>
+    <tableColumn id="7" xr3:uid="{208ABD57-DE4B-41D6-B9FC-93F2D8966E8D}" name="Letzter Wettkampf am" dataDxfId="79"/>
+    <tableColumn id="8" xr3:uid="{30C9697C-6550-4996-ADDB-7FEE5325B794}" name="Landesverband" dataDxfId="78"/>
+    <tableColumn id="9" xr3:uid="{ED2DAB77-EF46-4D8B-B8E4-90412E32E277}" name="OMS" dataDxfId="77"/>
+    <tableColumn id="10" xr3:uid="{AD534940-A91B-4A6E-9606-E3F3E517D401}" name="Pool-Länge" dataDxfId="76"/>
+    <tableColumn id="11" xr3:uid="{11F9D5D5-72FE-42CA-8624-01D513B4140F}" name="Regelwerk" dataDxfId="75"/>
+    <tableColumn id="12" xr3:uid="{3907872B-5438-4FBF-A045-3EF9EAACFC47}" name="Seiten Anzahl" dataDxfId="74"/>
+    <tableColumn id="13" xr3:uid="{FC821324-3638-40C0-BA1E-069B44E23C7A}" name="PZ1 - 50m Retten" dataDxfId="73"/>
+    <tableColumn id="14" xr3:uid="{70529619-443E-40D3-88C1-3E0F00BB2A50}" name="PZ1 - 100m Retten" dataDxfId="72"/>
+    <tableColumn id="15" xr3:uid="{EFA92FD2-C23F-42B3-83DC-5036513F19AF}" name="PZ1 - 100m Kombi" dataDxfId="71"/>
+    <tableColumn id="16" xr3:uid="{03309E52-8CF3-4E90-9EE6-A818901C3B32}" name="PZ1 - 100m Lifesaver" dataDxfId="70"/>
+    <tableColumn id="17" xr3:uid="{00B22013-AA11-4C17-9250-22060AE4B0A8}" name="PZ1 - 200m Super-Lifesaver" dataDxfId="69"/>
+    <tableColumn id="18" xr3:uid="{7E3508A9-0422-4561-A23E-53E613259B24}" name="PZ1 - 200m Hindernis" dataDxfId="68"/>
+    <tableColumn id="19" xr3:uid="{5CEA435F-F34B-4D8D-88D0-F5EBFF18B713}" name="PZ2 - 50m Retten" dataDxfId="67"/>
+    <tableColumn id="20" xr3:uid="{8585BE62-F7C4-4D5D-B287-052B43B08610}" name="PZ2 - 100m Retten" dataDxfId="66"/>
+    <tableColumn id="21" xr3:uid="{D981758B-ADAD-4E36-B787-0B0FDA808CA2}" name="PZ2 - 100m Kombi" dataDxfId="65"/>
+    <tableColumn id="22" xr3:uid="{1D4970A8-D22F-4962-934C-AEA295ED687A}" name="PZ2 - 100m Lifesaver" dataDxfId="64"/>
+    <tableColumn id="23" xr3:uid="{BE394430-C58F-4690-9615-44475E5AF9F8}" name="PZ2 - 200m Super-Lifesaver" dataDxfId="63"/>
+    <tableColumn id="24" xr3:uid="{A7036B1A-99CE-4F7C-AAB8-12E8B2696202}" name="PZ2 - 200m Hindernis" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}" name="LK_konfig" displayName="LK_konfig" ref="A1:AF37" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="A1:AF37" xr:uid="{FED162EE-531E-453F-8C25-562B59ECE709}"/>
   <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="52"/>
-    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="50"/>
-    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="48"/>
-    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="46"/>
-    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="45"/>
-    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="44"/>
-    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="43"/>
-    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="42"/>
-    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="41"/>
-    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="40"/>
-    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="39"/>
-    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="38"/>
-    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="37"/>
-    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="36"/>
-    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="35"/>
-    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="34"/>
-    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="33"/>
-    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="32"/>
-    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="31"/>
-    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="30"/>
-    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="29"/>
-    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="28"/>
-    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="27"/>
-    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{F985A4F0-6B8C-47C6-816F-1A31A4973EB2}" name="Tabellen Name" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{5E5AD859-71A2-4E8E-B434-431A89C05C57}" name="Geschlecht" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{85BB892C-E151-404B-8974-FC5199E0909C}" name="Mindest Alter" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{790F6CF9-E475-4082-AE03-D30EDE22FB61}" name="Maximales Alter" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{FD4B0E6E-9B64-4731-A50F-D3CE3A4ED3FC}" name="Qualizeitraum anfang" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{5E84CAD2-C403-49B9-BB06-D56EC5784C8C}" name="Qualizeitraum Ende" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{6323F8E2-5DA4-4E5B-9C35-1E8C219ADECF}" name="Letzter Wettkampf am" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{D2845930-152E-432F-92A0-E7F7A3EE1FF0}" name="Landesverband" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{87046373-5CCD-41EC-B34C-C753E71FD26C}" name="OMS" dataDxfId="51"/>
+    <tableColumn id="10" xr3:uid="{A685FE01-F23C-4533-B399-857F5A1F6C37}" name="Pool-Länge" dataDxfId="50"/>
+    <tableColumn id="11" xr3:uid="{11E0A508-0C9D-4CB6-952E-7FAC5D05BDCD}" name="Regelwerk" dataDxfId="49"/>
+    <tableColumn id="12" xr3:uid="{F220BD5F-C3B5-4935-996A-BFCDF9F392D9}" name="Seiten Anzahl" dataDxfId="48"/>
+    <tableColumn id="25" xr3:uid="{7CDE58FE-A5B8-4329-9F48-3913AEBA21FC}" name="mind. erreichte Normen" dataDxfId="47"/>
+    <tableColumn id="13" xr3:uid="{A0A5E62D-9354-426D-9A08-13E43F36F55B}" name="PZ - 50m Retten" dataDxfId="46"/>
+    <tableColumn id="14" xr3:uid="{5D70F54C-57E9-45E2-BC99-0DBB0422383E}" name="PZ - 100m Retten" dataDxfId="45"/>
+    <tableColumn id="15" xr3:uid="{1C0CF5DB-156E-4813-A8BA-9EA29A40ABF3}" name="PZ - 100m Kombi" dataDxfId="44"/>
+    <tableColumn id="16" xr3:uid="{691CD4E1-13D9-4455-A2D1-14C9BC41A0EA}" name="PZ - 100m Lifesaver" dataDxfId="43"/>
+    <tableColumn id="17" xr3:uid="{CE1BA235-770B-4FA4-B327-187675DDA6B8}" name="PZ - 200m Super-Lifesaver" dataDxfId="42"/>
+    <tableColumn id="18" xr3:uid="{A326EF87-5FF5-4042-85D3-7806FEED4CFA}" name="PZ - 200m Hindernis" dataDxfId="41"/>
+    <tableColumn id="19" xr3:uid="{3F3DF994-C8AE-408C-BCA1-99A143BA81D4}" name="LMS" dataDxfId="40"/>
+    <tableColumn id="20" xr3:uid="{7461FBF0-E903-4B09-9C11-C9C1047FA39D}" name="DMM" dataDxfId="39"/>
+    <tableColumn id="21" xr3:uid="{675AEE5F-BEC3-499A-A337-72DD69B663E7}" name="DEM" dataDxfId="38"/>
+    <tableColumn id="24" xr3:uid="{17E128CD-0800-40BC-B850-0CE3966127B2}" name="JRP" dataDxfId="37"/>
+    <tableColumn id="22" xr3:uid="{A92C8C64-1269-48FF-8F43-8EF273E7864F}" name="DMO" dataDxfId="36"/>
+    <tableColumn id="30" xr3:uid="{84286FAC-A077-44AC-889C-09543C869BF4}" name="DMO Ocean" dataDxfId="35"/>
+    <tableColumn id="23" xr3:uid="{40EF7D68-4E22-4866-ADAA-28DC8A82A09C}" name="Trophy" dataDxfId="34"/>
+    <tableColumn id="31" xr3:uid="{33F8EB16-27F6-453C-81FD-376213F45978}" name="Ocean Perf" dataDxfId="33"/>
+    <tableColumn id="32" xr3:uid="{5B81C846-FAFA-4E74-8678-47219E5942AF}" name="Filcow" dataDxfId="32"/>
+    <tableColumn id="26" xr3:uid="{C7421A01-D221-4C7A-9F0B-8BD025E0F1CF}" name="WM" dataDxfId="31"/>
+    <tableColumn id="27" xr3:uid="{4050AB9D-D7D4-4B88-8218-9206C91AD9A0}" name="EM" dataDxfId="30"/>
+    <tableColumn id="28" xr3:uid="{6FC272EA-276B-4249-818D-C220B87D52A6}" name="JWM" dataDxfId="29"/>
+    <tableColumn id="29" xr3:uid="{51F99A1A-8D2C-444F-9E7C-AA537C8FFA08}" name="JEM" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8772,52 +8782,52 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5:G31">
-    <cfRule type="expression" dxfId="20" priority="15">
+    <cfRule type="expression" dxfId="22" priority="15">
       <formula>B5&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:M31">
-    <cfRule type="expression" dxfId="19" priority="14">
+    <cfRule type="expression" dxfId="21" priority="14">
       <formula>H5&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:S31">
-    <cfRule type="expression" dxfId="18" priority="13">
+    <cfRule type="expression" dxfId="20" priority="13">
       <formula>N5&lt;&gt;N4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:Y31">
-    <cfRule type="expression" dxfId="17" priority="12">
+    <cfRule type="expression" dxfId="19" priority="12">
       <formula>T5&lt;&gt;T4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z5:AE31">
-    <cfRule type="expression" dxfId="16" priority="9">
+    <cfRule type="expression" dxfId="18" priority="9">
       <formula>Z5&lt;&gt;Z4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF5:AK31">
-    <cfRule type="expression" dxfId="15" priority="8">
+    <cfRule type="expression" dxfId="17" priority="8">
       <formula>AF5&lt;&gt;AF4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL5:AN31">
-    <cfRule type="expression" dxfId="14" priority="6">
+    <cfRule type="expression" dxfId="16" priority="6">
       <formula>AL5&lt;&gt;AL4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO5:AQ31">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>AO5&lt;&gt;AO4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR5:AT31">
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>AR5&lt;&gt;AR4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU5:AW31">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>AU5&lt;&gt;AU4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8846,133 +8856,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:78" s="39" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="125">
+      <c r="A1" s="108">
         <v>2025</v>
       </c>
       <c r="B1" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="106" t="s">
+      <c r="C1" s="109" t="s">
         <v>209</v>
       </c>
-      <c r="D1" s="106"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="110" t="s">
+      <c r="D1" s="109"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="111" t="s">
         <v>210</v>
       </c>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="116" t="s">
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="114" t="s">
         <v>214</v>
       </c>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="108" t="s">
+      <c r="L1" s="115"/>
+      <c r="M1" s="115"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="134" t="s">
         <v>211</v>
       </c>
-      <c r="P1" s="108"/>
-      <c r="Q1" s="109"/>
-      <c r="R1" s="122" t="s">
+      <c r="P1" s="134"/>
+      <c r="Q1" s="135"/>
+      <c r="R1" s="136" t="s">
         <v>212</v>
       </c>
-      <c r="S1" s="123"/>
-      <c r="T1" s="123"/>
-      <c r="U1" s="123"/>
-      <c r="V1" s="124"/>
-      <c r="W1" s="119" t="s">
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="138"/>
+      <c r="W1" s="139" t="s">
         <v>215</v>
       </c>
-      <c r="X1" s="120"/>
-      <c r="Y1" s="120"/>
-      <c r="Z1" s="121"/>
+      <c r="X1" s="140"/>
+      <c r="Y1" s="140"/>
+      <c r="Z1" s="141"/>
       <c r="AA1"/>
       <c r="AB1" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="126" t="s">
+      <c r="AC1" s="117" t="s">
         <v>216</v>
       </c>
-      <c r="AD1" s="126"/>
-      <c r="AE1" s="127"/>
-      <c r="AF1" s="128" t="s">
+      <c r="AD1" s="117"/>
+      <c r="AE1" s="118"/>
+      <c r="AF1" s="119" t="s">
         <v>217</v>
       </c>
-      <c r="AG1" s="129"/>
-      <c r="AH1" s="129"/>
-      <c r="AI1" s="129"/>
-      <c r="AJ1" s="130"/>
-      <c r="AK1" s="131" t="s">
+      <c r="AG1" s="120"/>
+      <c r="AH1" s="120"/>
+      <c r="AI1" s="120"/>
+      <c r="AJ1" s="121"/>
+      <c r="AK1" s="122" t="s">
         <v>218</v>
       </c>
-      <c r="AL1" s="132"/>
-      <c r="AM1" s="132"/>
-      <c r="AN1" s="133"/>
-      <c r="AO1" s="134" t="s">
+      <c r="AL1" s="123"/>
+      <c r="AM1" s="123"/>
+      <c r="AN1" s="124"/>
+      <c r="AO1" s="125" t="s">
         <v>219</v>
       </c>
-      <c r="AP1" s="135"/>
-      <c r="AQ1" s="136"/>
-      <c r="AR1" s="137" t="s">
+      <c r="AP1" s="126"/>
+      <c r="AQ1" s="127"/>
+      <c r="AR1" s="128" t="s">
         <v>220</v>
       </c>
-      <c r="AS1" s="138"/>
-      <c r="AT1" s="138"/>
-      <c r="AU1" s="138"/>
-      <c r="AV1" s="139"/>
-      <c r="AW1" s="113" t="s">
+      <c r="AS1" s="129"/>
+      <c r="AT1" s="129"/>
+      <c r="AU1" s="129"/>
+      <c r="AV1" s="130"/>
+      <c r="AW1" s="131" t="s">
         <v>221</v>
       </c>
-      <c r="AX1" s="114"/>
-      <c r="AY1" s="114"/>
-      <c r="AZ1" s="115"/>
+      <c r="AX1" s="132"/>
+      <c r="AY1" s="132"/>
+      <c r="AZ1" s="133"/>
       <c r="BB1" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="106" t="s">
+      <c r="BC1" s="109" t="s">
         <v>222</v>
       </c>
-      <c r="BD1" s="106"/>
-      <c r="BE1" s="107"/>
-      <c r="BF1" s="110" t="s">
+      <c r="BD1" s="109"/>
+      <c r="BE1" s="110"/>
+      <c r="BF1" s="111" t="s">
         <v>223</v>
       </c>
-      <c r="BG1" s="111"/>
-      <c r="BH1" s="111"/>
-      <c r="BI1" s="111"/>
-      <c r="BJ1" s="112"/>
-      <c r="BK1" s="116" t="s">
+      <c r="BG1" s="112"/>
+      <c r="BH1" s="112"/>
+      <c r="BI1" s="112"/>
+      <c r="BJ1" s="113"/>
+      <c r="BK1" s="114" t="s">
         <v>224</v>
       </c>
-      <c r="BL1" s="117"/>
-      <c r="BM1" s="117"/>
-      <c r="BN1" s="118"/>
-      <c r="BO1" s="108" t="s">
+      <c r="BL1" s="115"/>
+      <c r="BM1" s="115"/>
+      <c r="BN1" s="116"/>
+      <c r="BO1" s="134" t="s">
         <v>229</v>
       </c>
-      <c r="BP1" s="108"/>
-      <c r="BQ1" s="109"/>
-      <c r="BR1" s="122" t="s">
+      <c r="BP1" s="134"/>
+      <c r="BQ1" s="135"/>
+      <c r="BR1" s="136" t="s">
         <v>230</v>
       </c>
-      <c r="BS1" s="123"/>
-      <c r="BT1" s="123"/>
-      <c r="BU1" s="123"/>
-      <c r="BV1" s="124"/>
-      <c r="BW1" s="119" t="s">
+      <c r="BS1" s="137"/>
+      <c r="BT1" s="137"/>
+      <c r="BU1" s="137"/>
+      <c r="BV1" s="138"/>
+      <c r="BW1" s="139" t="s">
         <v>225</v>
       </c>
-      <c r="BX1" s="120"/>
-      <c r="BY1" s="120"/>
-      <c r="BZ1" s="121"/>
+      <c r="BX1" s="140"/>
+      <c r="BY1" s="140"/>
+      <c r="BZ1" s="141"/>
     </row>
     <row r="2" spans="1:78" s="93" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="125"/>
+      <c r="A2" s="108"/>
       <c r="B2" s="45" t="s">
         <v>213</v>
       </c>
@@ -9273,7 +9283,7 @@
       </c>
     </row>
     <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="125"/>
+      <c r="A3" s="108"/>
       <c r="B3" s="46" t="s">
         <v>0</v>
       </c>
@@ -9526,7 +9536,7 @@
       </c>
     </row>
     <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="125"/>
+      <c r="A4" s="108"/>
       <c r="B4" s="46" t="s">
         <v>181</v>
       </c>
@@ -9778,7 +9788,7 @@
       </c>
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="125"/>
+      <c r="A5" s="108"/>
       <c r="B5" s="46" t="s">
         <v>182</v>
       </c>
@@ -10030,7 +10040,7 @@
       </c>
     </row>
     <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="125"/>
+      <c r="A6" s="108"/>
       <c r="B6" s="46" t="s">
         <v>183</v>
       </c>
@@ -10282,7 +10292,7 @@
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="125"/>
+      <c r="A7" s="108"/>
       <c r="B7" s="46" t="s">
         <v>184</v>
       </c>
@@ -10534,7 +10544,7 @@
       </c>
     </row>
     <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="125"/>
+      <c r="A8" s="108"/>
       <c r="B8" s="49" t="s">
         <v>4</v>
       </c>
@@ -10787,132 +10797,132 @@
     </row>
     <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="125">
+      <c r="A10" s="108">
         <v>2026</v>
       </c>
       <c r="B10" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="106" t="s">
+      <c r="C10" s="109" t="s">
         <v>209</v>
       </c>
-      <c r="D10" s="106"/>
-      <c r="E10" s="107"/>
-      <c r="F10" s="110" t="s">
+      <c r="D10" s="109"/>
+      <c r="E10" s="110"/>
+      <c r="F10" s="111" t="s">
         <v>210</v>
       </c>
-      <c r="G10" s="111"/>
-      <c r="H10" s="111"/>
-      <c r="I10" s="111"/>
-      <c r="J10" s="112"/>
-      <c r="K10" s="116" t="s">
+      <c r="G10" s="112"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+      <c r="J10" s="113"/>
+      <c r="K10" s="114" t="s">
         <v>214</v>
       </c>
-      <c r="L10" s="117"/>
-      <c r="M10" s="117"/>
-      <c r="N10" s="118"/>
-      <c r="O10" s="108" t="s">
+      <c r="L10" s="115"/>
+      <c r="M10" s="115"/>
+      <c r="N10" s="116"/>
+      <c r="O10" s="134" t="s">
         <v>211</v>
       </c>
-      <c r="P10" s="108"/>
-      <c r="Q10" s="109"/>
-      <c r="R10" s="122" t="s">
+      <c r="P10" s="134"/>
+      <c r="Q10" s="135"/>
+      <c r="R10" s="136" t="s">
         <v>212</v>
       </c>
-      <c r="S10" s="123"/>
-      <c r="T10" s="123"/>
-      <c r="U10" s="123"/>
-      <c r="V10" s="124"/>
-      <c r="W10" s="119" t="s">
+      <c r="S10" s="137"/>
+      <c r="T10" s="137"/>
+      <c r="U10" s="137"/>
+      <c r="V10" s="138"/>
+      <c r="W10" s="139" t="s">
         <v>215</v>
       </c>
-      <c r="X10" s="120"/>
-      <c r="Y10" s="120"/>
-      <c r="Z10" s="121"/>
+      <c r="X10" s="140"/>
+      <c r="Y10" s="140"/>
+      <c r="Z10" s="141"/>
       <c r="AB10" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="126" t="s">
+      <c r="AC10" s="117" t="s">
         <v>216</v>
       </c>
-      <c r="AD10" s="126"/>
-      <c r="AE10" s="127"/>
-      <c r="AF10" s="128" t="s">
+      <c r="AD10" s="117"/>
+      <c r="AE10" s="118"/>
+      <c r="AF10" s="119" t="s">
         <v>217</v>
       </c>
-      <c r="AG10" s="129"/>
-      <c r="AH10" s="129"/>
-      <c r="AI10" s="129"/>
-      <c r="AJ10" s="130"/>
-      <c r="AK10" s="131" t="s">
+      <c r="AG10" s="120"/>
+      <c r="AH10" s="120"/>
+      <c r="AI10" s="120"/>
+      <c r="AJ10" s="121"/>
+      <c r="AK10" s="122" t="s">
         <v>218</v>
       </c>
-      <c r="AL10" s="132"/>
-      <c r="AM10" s="132"/>
-      <c r="AN10" s="133"/>
-      <c r="AO10" s="134" t="s">
+      <c r="AL10" s="123"/>
+      <c r="AM10" s="123"/>
+      <c r="AN10" s="124"/>
+      <c r="AO10" s="125" t="s">
         <v>219</v>
       </c>
-      <c r="AP10" s="135"/>
-      <c r="AQ10" s="136"/>
-      <c r="AR10" s="137" t="s">
+      <c r="AP10" s="126"/>
+      <c r="AQ10" s="127"/>
+      <c r="AR10" s="128" t="s">
         <v>220</v>
       </c>
-      <c r="AS10" s="138"/>
-      <c r="AT10" s="138"/>
-      <c r="AU10" s="138"/>
-      <c r="AV10" s="139"/>
-      <c r="AW10" s="113" t="s">
+      <c r="AS10" s="129"/>
+      <c r="AT10" s="129"/>
+      <c r="AU10" s="129"/>
+      <c r="AV10" s="130"/>
+      <c r="AW10" s="131" t="s">
         <v>221</v>
       </c>
-      <c r="AX10" s="114"/>
-      <c r="AY10" s="114"/>
-      <c r="AZ10" s="115"/>
+      <c r="AX10" s="132"/>
+      <c r="AY10" s="132"/>
+      <c r="AZ10" s="133"/>
       <c r="BB10" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="106" t="s">
+      <c r="BC10" s="109" t="s">
         <v>222</v>
       </c>
-      <c r="BD10" s="106"/>
-      <c r="BE10" s="107"/>
-      <c r="BF10" s="110" t="s">
+      <c r="BD10" s="109"/>
+      <c r="BE10" s="110"/>
+      <c r="BF10" s="111" t="s">
         <v>223</v>
       </c>
-      <c r="BG10" s="111"/>
-      <c r="BH10" s="111"/>
-      <c r="BI10" s="111"/>
-      <c r="BJ10" s="112"/>
-      <c r="BK10" s="116" t="s">
+      <c r="BG10" s="112"/>
+      <c r="BH10" s="112"/>
+      <c r="BI10" s="112"/>
+      <c r="BJ10" s="113"/>
+      <c r="BK10" s="114" t="s">
         <v>224</v>
       </c>
-      <c r="BL10" s="117"/>
-      <c r="BM10" s="117"/>
-      <c r="BN10" s="118"/>
-      <c r="BO10" s="108" t="s">
+      <c r="BL10" s="115"/>
+      <c r="BM10" s="115"/>
+      <c r="BN10" s="116"/>
+      <c r="BO10" s="134" t="s">
         <v>229</v>
       </c>
-      <c r="BP10" s="108"/>
-      <c r="BQ10" s="109"/>
-      <c r="BR10" s="122" t="s">
+      <c r="BP10" s="134"/>
+      <c r="BQ10" s="135"/>
+      <c r="BR10" s="136" t="s">
         <v>230</v>
       </c>
-      <c r="BS10" s="123"/>
-      <c r="BT10" s="123"/>
-      <c r="BU10" s="123"/>
-      <c r="BV10" s="124"/>
-      <c r="BW10" s="119" t="s">
+      <c r="BS10" s="137"/>
+      <c r="BT10" s="137"/>
+      <c r="BU10" s="137"/>
+      <c r="BV10" s="138"/>
+      <c r="BW10" s="139" t="s">
         <v>225</v>
       </c>
-      <c r="BX10" s="120"/>
-      <c r="BY10" s="120"/>
-      <c r="BZ10" s="121"/>
+      <c r="BX10" s="140"/>
+      <c r="BY10" s="140"/>
+      <c r="BZ10" s="141"/>
     </row>
     <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="125"/>
+      <c r="A11" s="108"/>
       <c r="B11" s="45" t="s">
         <v>213</v>
       </c>
@@ -11213,7 +11223,7 @@
       </c>
     </row>
     <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="125"/>
+      <c r="A12" s="108"/>
       <c r="B12" s="46" t="s">
         <v>0</v>
       </c>
@@ -11465,7 +11475,7 @@
       </c>
     </row>
     <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="125"/>
+      <c r="A13" s="108"/>
       <c r="B13" s="46" t="s">
         <v>181</v>
       </c>
@@ -11717,7 +11727,7 @@
       </c>
     </row>
     <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="125"/>
+      <c r="A14" s="108"/>
       <c r="B14" s="46" t="s">
         <v>182</v>
       </c>
@@ -11969,7 +11979,7 @@
       </c>
     </row>
     <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="125"/>
+      <c r="A15" s="108"/>
       <c r="B15" s="46" t="s">
         <v>183</v>
       </c>
@@ -12221,7 +12231,7 @@
       </c>
     </row>
     <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="125"/>
+      <c r="A16" s="108"/>
       <c r="B16" s="46" t="s">
         <v>184</v>
       </c>
@@ -12473,7 +12483,7 @@
       </c>
     </row>
     <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="125"/>
+      <c r="A17" s="108"/>
       <c r="B17" s="49" t="s">
         <v>4</v>
       </c>
@@ -12940,6 +12950,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -12956,36 +12988,14 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC12:AZ17">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13308,7 +13318,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:H14">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>$A2&lt;TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14314,22 +14324,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="10" priority="20">
+    <cfRule type="expression" dxfId="12" priority="20">
       <formula>B6&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>B7&lt;&gt;B6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="8" priority="22">
+    <cfRule type="expression" dxfId="10" priority="22">
       <formula>H6&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="9" priority="2">
       <formula>H7&lt;&gt;H6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14545,14 +14555,14 @@
       <c r="I5" s="4">
         <v>6.0335648148148152E-4</v>
       </c>
-      <c r="J5" s="141">
+      <c r="J5" s="107">
         <v>7.8541666666666668E-4</v>
       </c>
-      <c r="K5" s="141">
+      <c r="K5" s="107">
         <v>6.4687499999999999E-4</v>
       </c>
-      <c r="L5" s="140"/>
-      <c r="M5" s="141">
+      <c r="L5" s="106"/>
+      <c r="M5" s="107">
         <v>8.7685185185185186E-4</v>
       </c>
     </row>
@@ -14577,7 +14587,9 @@
       <c r="G6" s="5">
         <v>1.5353009259259261E-3</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" s="3">
+        <v>3.8425925925925927E-4</v>
+      </c>
       <c r="I6" s="3">
         <v>6.0335648148148152E-4</v>
       </c>
@@ -14603,7 +14615,7 @@
         <v>4.5000000000000004E-4</v>
       </c>
       <c r="C7" s="4">
-        <v>6.864583333333333E-4</v>
+        <v>7.0497685185185192E-4</v>
       </c>
       <c r="D7" s="4">
         <v>9.1134259259259261E-4</v>
@@ -14645,7 +14657,7 @@
         <v>4.1504629629629633E-4</v>
       </c>
       <c r="C8" s="3">
-        <v>6.9363425925925929E-4</v>
+        <v>6.8645833333333341E-4</v>
       </c>
       <c r="D8" s="3">
         <v>8.6585648148148166E-4</v>
@@ -14687,7 +14699,7 @@
         <v>4.1446759259259258E-4</v>
       </c>
       <c r="C9" s="4">
-        <v>6.9363425925925929E-4</v>
+        <v>6.5891203703703706E-4</v>
       </c>
       <c r="D9" s="4">
         <v>8.6585648148148166E-4</v>
@@ -14729,7 +14741,7 @@
         <v>4.130787037037037E-4</v>
       </c>
       <c r="C10" s="3">
-        <v>6.9363425925925929E-4</v>
+        <v>6.5891203703703706E-4</v>
       </c>
       <c r="D10" s="3">
         <v>8.524305555555556E-4</v>
@@ -14771,7 +14783,7 @@
         <v>4.1203703703703709E-4</v>
       </c>
       <c r="C11" s="4">
-        <v>6.9363425925925929E-4</v>
+        <v>6.5891203703703706E-4</v>
       </c>
       <c r="D11" s="4">
         <v>8.524305555555556E-4</v>
@@ -15687,24 +15699,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:G6">
-    <cfRule type="expression" dxfId="6" priority="19">
-      <formula>B6&lt;&gt;B4</formula>
+  <conditionalFormatting sqref="B5:G32">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>B5&lt;&gt;B4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:G32">
-    <cfRule type="expression" dxfId="5" priority="2">
-      <formula>B7&lt;&gt;B6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H6:M6">
-    <cfRule type="expression" dxfId="4" priority="20">
-      <formula>H6&lt;&gt;H4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:M32">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>H7&lt;&gt;H6</formula>
+  <conditionalFormatting sqref="H5:M32">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>H5&lt;&gt;H4</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
NEW JRP Records Krit
</commit_message>
<xml_diff>
--- a/web/data/records_kriterien.xlsx
+++ b/web/data/records_kriterien.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpgna\Documents\GitHub\Lifesaving_Baden\web\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8989B893-329E-45F7-A665-2B46637A0875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C32FA5-24B5-4309-812D-C1F4AB6FBAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" activeTab="1" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="687" activeTab="7" xr2:uid="{E1AB626B-3773-4829-92A5-28DD4DB7C8F8}"/>
   </bookViews>
   <sheets>
     <sheet name="DR" sheetId="9" r:id="rId1"/>
@@ -1707,16 +1707,13 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1728,15 +1725,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1745,27 +1733,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1809,6 +1776,39 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
@@ -2440,110 +2440,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="m:ss.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2797,31 +2693,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="medium">
           <color theme="0"/>
@@ -4215,16 +4086,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="medium">
-          <color theme="3" tint="-0.499984740745262"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -4329,6 +4190,16 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color theme="3" tint="-0.499984740745262"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -4358,6 +4229,110 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="m:ss.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -4387,6 +4362,31 @@
           <color theme="3" tint="-0.499984740745262"/>
         </right>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -4434,60 +4434,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="244" headerRowBorderDxfId="243" tableBorderDxfId="242">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}" name="WR_Open4" displayName="WR_Open4" ref="A4:AW31" totalsRowShown="0" headerRowDxfId="239" headerRowBorderDxfId="238" tableBorderDxfId="237">
   <autoFilter ref="A4:AW31" xr:uid="{2C5E83EE-6B6F-478A-9C90-A846A1A76536}"/>
   <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="241">
+    <tableColumn id="1" xr3:uid="{7C0C4105-A61A-4B8D-9129-EDC4F18765AF}" name="WR-Open" dataDxfId="236">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="240"/>
-    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="239"/>
-    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="238"/>
-    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="237"/>
-    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="236"/>
-    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="235"/>
-    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="234"/>
-    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="233"/>
+    <tableColumn id="2" xr3:uid="{516F5612-F85F-413F-9012-E235F415E34B}" name="50m Retten - offen - W" dataDxfId="235"/>
+    <tableColumn id="3" xr3:uid="{BC9ACAC9-0D45-42FD-B596-D19FBE3A4D83}" name="100m Retten - offen - W" dataDxfId="234"/>
+    <tableColumn id="4" xr3:uid="{CB6DBE59-EB65-43F0-93E7-0BDC3F82832B}" name="100m Kombi - offen - W" dataDxfId="233"/>
+    <tableColumn id="5" xr3:uid="{AA603C60-6831-4C14-A8CD-0AA050DA7551}" name="100m Lifesaver - offen - W" dataDxfId="232"/>
+    <tableColumn id="6" xr3:uid="{7920F147-7717-4582-940A-2610F7D310CA}" name="200m Superlifesaver - offen - W" dataDxfId="231"/>
+    <tableColumn id="7" xr3:uid="{04E21F1D-AC8D-4A1B-9B43-59B8F7901673}" name="200m Hindernis - offen - W" dataDxfId="230"/>
+    <tableColumn id="8" xr3:uid="{40E8A083-653A-48A8-9B37-0A2D850B7829}" name="50m Retten - offen - M" dataDxfId="229"/>
+    <tableColumn id="9" xr3:uid="{863824A9-134F-4189-BB14-225AE224FC44}" name="100m Retten - offen - M" dataDxfId="228"/>
     <tableColumn id="10" xr3:uid="{598FC6AE-DEA2-4475-9A35-CDCB8C81496A}" name="100m Kombi - offen - M"/>
     <tableColumn id="11" xr3:uid="{9FC50B37-0D51-422E-A268-A6506D4F3854}" name="100m Lifesaver - offen - M"/>
     <tableColumn id="12" xr3:uid="{B8D2552B-5D82-442A-98F0-E47D5C5F6728}" name="200m Superlifesaver - offen - M"/>
-    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="232"/>
-    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="231"/>
-    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="230"/>
-    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="229"/>
-    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="228"/>
-    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="227"/>
-    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="226"/>
-    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="225"/>
-    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="224"/>
-    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="223"/>
-    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="222"/>
-    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="221"/>
-    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="220"/>
-    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="219"/>
-    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="218"/>
-    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="217"/>
-    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="216"/>
-    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="215"/>
-    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="214"/>
-    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="213"/>
-    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="212"/>
-    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="211"/>
-    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="210"/>
-    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="209"/>
-    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="208"/>
-    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="207"/>
-    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="206"/>
-    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="205"/>
-    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="204"/>
-    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="203"/>
-    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="202"/>
-    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="201"/>
-    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="200"/>
-    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="199"/>
-    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="198"/>
-    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="197"/>
-    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="196"/>
+    <tableColumn id="13" xr3:uid="{5A5E9873-0C5F-4508-AF6B-4974E0526D84}" name="200m Hindernis - offen - M" dataDxfId="227"/>
+    <tableColumn id="14" xr3:uid="{FA907992-7FCE-4CAD-8CF2-F5BEBC9B3756}" name="50m Retten - 17/18 - W" dataDxfId="226"/>
+    <tableColumn id="15" xr3:uid="{76B63DC0-CB67-48F4-9B5A-D22902F59334}" name="100m Retten - 17/18 - W" dataDxfId="225"/>
+    <tableColumn id="16" xr3:uid="{614A2419-51B1-44C0-8469-ADBFB078B81A}" name="100m Kombi -17/18 - W" dataDxfId="224"/>
+    <tableColumn id="17" xr3:uid="{2EC953EE-367D-4524-A25E-8DE3B8168E34}" name="100m Lifesaver - 17/18 - W" dataDxfId="223"/>
+    <tableColumn id="18" xr3:uid="{25711867-9BD7-4197-9094-A21392411249}" name="200m Superlifesaver - 17/18 - W" dataDxfId="222"/>
+    <tableColumn id="19" xr3:uid="{262DB142-CFB1-45C3-9332-7273CACD1B62}" name="200m Hindernis - 17/18 - W" dataDxfId="221"/>
+    <tableColumn id="20" xr3:uid="{938BA45A-8244-4637-8A14-DF49CD91A945}" name="50m Retten - 17/18 - M" dataDxfId="220"/>
+    <tableColumn id="21" xr3:uid="{737E28D8-900F-4A98-95FE-EE7B0AFDEE90}" name="100m Retten - 17/18 - M" dataDxfId="219"/>
+    <tableColumn id="22" xr3:uid="{330BD3A8-061C-45E2-ADDB-40C2F346772F}" name="100m Kombi - 17/18 - M" dataDxfId="218"/>
+    <tableColumn id="23" xr3:uid="{0CADDE90-A167-4E1D-8D33-8624E5E1A4E2}" name="100m Lifesaver - 17/18 - M" dataDxfId="217"/>
+    <tableColumn id="24" xr3:uid="{FCF9F42C-1291-4985-9D37-B9DE2DAA5DCB}" name="200m Superlifesaver - 17/18 - M" dataDxfId="216"/>
+    <tableColumn id="25" xr3:uid="{4E5397B2-F924-4F48-AE69-AF6D650AF88D}" name="200m Hindernis - 17/18 - M" dataDxfId="215"/>
+    <tableColumn id="26" xr3:uid="{0A78315A-BFDC-43EE-A66F-48B301F66508}" name="50m Retten - 15/16 - W" dataDxfId="214"/>
+    <tableColumn id="27" xr3:uid="{D3FCF8BD-6C76-450D-80C0-CC0519A79731}" name="100m Retten - 15/16 - W" dataDxfId="213"/>
+    <tableColumn id="28" xr3:uid="{6BE7937E-D62D-47CD-95DE-1730304B0DF3}" name="100m Kombi - 15/16 - W" dataDxfId="212"/>
+    <tableColumn id="29" xr3:uid="{098BA5BE-5AF6-4187-89B6-534498F24C51}" name="100m Lifesaver -  15/16 - W" dataDxfId="211"/>
+    <tableColumn id="30" xr3:uid="{2A6822CF-143C-4BF7-A440-5777527BE512}" name="200m Superlifesaver -  15/16 - W" dataDxfId="210"/>
+    <tableColumn id="31" xr3:uid="{541C7145-CDEA-4E4E-9E7A-A4F05BA6C3E5}" name="200m Hindernis -  15/16 - W" dataDxfId="209"/>
+    <tableColumn id="32" xr3:uid="{342C4488-8C61-42E6-87A9-C75BD8EB7452}" name="50m Retten - 15/16 - M" dataDxfId="208"/>
+    <tableColumn id="33" xr3:uid="{857B1D46-7D20-47F7-AB9B-732D50346E32}" name="100m Retten - 15/16 - M" dataDxfId="207"/>
+    <tableColumn id="34" xr3:uid="{4C8A2EB4-804B-45F1-A768-9A6958957F8B}" name="100m Kombi -15/16 - M" dataDxfId="206"/>
+    <tableColumn id="35" xr3:uid="{26C75B4F-21EC-4EB0-A9A9-54BC80140672}" name="100m Lifesaver - 15/16 - M" dataDxfId="205"/>
+    <tableColumn id="36" xr3:uid="{DBBB2A23-1A06-429A-A5D1-A547EF5EC16F}" name="200m Superlifesaver - 15/16 - M" dataDxfId="204"/>
+    <tableColumn id="37" xr3:uid="{84061231-CAE5-427A-87F5-6DDBA99F77D2}" name="200m Hindernis - 15/16 - M" dataDxfId="203"/>
+    <tableColumn id="38" xr3:uid="{878CCA80-A742-4B3C-90C9-E93BB814201B}" name="50m Retten - 13/14 - W" dataDxfId="202"/>
+    <tableColumn id="39" xr3:uid="{A1F57102-61CF-4784-8DE2-0B8F32D5D699}" name="50m Retten mit Flossen - 13/14 - W" dataDxfId="201"/>
+    <tableColumn id="40" xr3:uid="{0F6BAF78-3D79-42A9-9FED-E6D0E335A920}" name="100m Hindernis - 13/14 - W" dataDxfId="200"/>
+    <tableColumn id="41" xr3:uid="{EB748A68-E10D-4D76-B315-8FDB3AC33C8D}" name="50m Retten - 13/14 - M" dataDxfId="199"/>
+    <tableColumn id="42" xr3:uid="{C7B04167-6430-40F0-9A0F-D0D0BE2F9C77}" name="50m Retten mit Flossen - 13/14 - M" dataDxfId="198"/>
+    <tableColumn id="43" xr3:uid="{48704BB7-A853-445A-8CDC-8D8F86C2B66A}" name="100m Hindernis - 13/14 - M" dataDxfId="197"/>
+    <tableColumn id="44" xr3:uid="{9605FE9A-F41C-4A5F-A59C-B7A9D45C460F}" name="50m Flossen - 12 - W" dataDxfId="196"/>
+    <tableColumn id="45" xr3:uid="{4C9DBF61-35B1-4BC2-8272-526E0AFAAFFB}" name="50m komb. Schwimmen - 12 - W" dataDxfId="195"/>
+    <tableColumn id="46" xr3:uid="{CF433C95-C272-48F9-98CD-7E3C8DBB6F2C}" name="50m Hindernis - 12 - W" dataDxfId="194"/>
+    <tableColumn id="47" xr3:uid="{FADB7411-DB43-4B14-B9E8-D74CA1BA18B8}" name="50m Flossen - 12 - M" dataDxfId="193"/>
+    <tableColumn id="48" xr3:uid="{02936F84-1D82-48AC-8D7C-6D2954D68A06}" name="50m komb. Schwimmen - 12 - M" dataDxfId="192"/>
+    <tableColumn id="49" xr3:uid="{7FD9BD11-0597-4E07-8DA5-DB53384197F5}" name="50m Hindernis - 12 - M" dataDxfId="191"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4511,42 +4511,42 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="195" dataDxfId="193" headerRowBorderDxfId="194" tableBorderDxfId="192">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}" name="WR_Youth" displayName="WR_Youth" ref="A4:M32" totalsRowShown="0" headerRowDxfId="256" dataDxfId="254" headerRowBorderDxfId="255" tableBorderDxfId="253">
   <autoFilter ref="A4:M32" xr:uid="{4234D44E-A2BE-4790-B589-1A8CC19B714E}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="191"/>
-    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="190"/>
-    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="189"/>
-    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="188"/>
-    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="187"/>
-    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="186"/>
-    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="185"/>
-    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="184"/>
-    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="183"/>
-    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="182"/>
-    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="181"/>
-    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="180"/>
-    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="179"/>
+    <tableColumn id="1" xr3:uid="{848E691A-41B0-42DD-B122-FB6DF43CB3EF}" name="WR-Youth" dataDxfId="252"/>
+    <tableColumn id="2" xr3:uid="{2FE43F18-485B-46A9-8946-FBC5FDAE5A8E}" name="50m Retten" dataDxfId="251"/>
+    <tableColumn id="3" xr3:uid="{CA5C3ABF-02E6-442B-868B-95B293B231D3}" name="100m Retten" dataDxfId="250"/>
+    <tableColumn id="4" xr3:uid="{7A6BBA52-2145-464D-8C04-B2CCFC1A90DC}" name="100m Kombi" dataDxfId="249"/>
+    <tableColumn id="5" xr3:uid="{21F420C9-E788-49EE-88F6-E37963ED31CF}" name="100m Lifesaver" dataDxfId="248"/>
+    <tableColumn id="6" xr3:uid="{CB87B7CD-8A9C-4775-A4D7-4D267F43FD1A}" name="200m Superlifesaver" dataDxfId="247"/>
+    <tableColumn id="7" xr3:uid="{2DC7F290-B564-4851-85AE-D211DA701B32}" name="200m Hindernis" dataDxfId="246"/>
+    <tableColumn id="8" xr3:uid="{8112783D-8796-4D6A-8414-AC675D745697}" name="50m Retten2" dataDxfId="245"/>
+    <tableColumn id="9" xr3:uid="{4E818CD4-8725-495D-9D1D-1AFCED9181F5}" name="100m Retten2" dataDxfId="244"/>
+    <tableColumn id="10" xr3:uid="{28C05A91-E302-40A9-B50A-ECF997F129FC}" name="100m Kombi2" dataDxfId="243"/>
+    <tableColumn id="11" xr3:uid="{D56FB9F2-45BF-4EC9-A84C-8A5FB59F2F05}" name="100m Lifesaver2" dataDxfId="242"/>
+    <tableColumn id="12" xr3:uid="{540169C0-2A40-4794-A872-F7DF8A887BF2}" name="200m Superlifesaver2" dataDxfId="241"/>
+    <tableColumn id="13" xr3:uid="{D104CB67-B55A-4C81-87E5-0AC758DD22A4}" name="200m Hindernis2" dataDxfId="240"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="256" headerRowBorderDxfId="255" tableBorderDxfId="254">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}" name="WR_Open" displayName="WR_Open" ref="A4:M32" totalsRowShown="0" headerRowDxfId="190" headerRowBorderDxfId="189" tableBorderDxfId="188">
   <autoFilter ref="A4:M32" xr:uid="{E2D2F97B-7645-4066-8AB3-F35CF6E035EB}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="253">
+    <tableColumn id="1" xr3:uid="{AE73402B-B27E-4B29-8DCF-30B7FC1855EF}" name="WR-Open" dataDxfId="187">
       <calculatedColumnFormula>A4+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="252"/>
-    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="251"/>
-    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="250"/>
-    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="249"/>
-    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="248"/>
-    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="247"/>
-    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="246"/>
-    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="245"/>
+    <tableColumn id="2" xr3:uid="{EA3EAC1F-184E-4A28-B3E3-08DE12F138EF}" name="50m Retten" dataDxfId="186"/>
+    <tableColumn id="3" xr3:uid="{E0305A3F-6087-4F8C-8B64-153E1ACAA32E}" name="100m Retten" dataDxfId="185"/>
+    <tableColumn id="4" xr3:uid="{F0B7AC37-315E-49AA-855C-7955D2B43A76}" name="100m Kombi" dataDxfId="184"/>
+    <tableColumn id="5" xr3:uid="{B5E690AB-DB7D-4864-8916-89D2A68C4128}" name="100m Lifesaver" dataDxfId="183"/>
+    <tableColumn id="6" xr3:uid="{D89BAF4D-36AE-4C73-9320-9C5736F02F8A}" name="200m Superlifesaver" dataDxfId="182"/>
+    <tableColumn id="7" xr3:uid="{58AE7517-1A90-459F-A7D2-B95265D217E7}" name="200m Hindernis" dataDxfId="181"/>
+    <tableColumn id="8" xr3:uid="{13A189FB-E897-4A1F-A001-525F61E9CFFF}" name="50m Retten2" dataDxfId="180"/>
+    <tableColumn id="9" xr3:uid="{36418AC5-46B8-400F-BD2E-D329CF4F92CD}" name="100m Retten2" dataDxfId="179"/>
     <tableColumn id="10" xr3:uid="{06A35C2D-7313-472B-BC1F-4F2FB1D14782}" name="100m Kombi2"/>
     <tableColumn id="11" xr3:uid="{89966D0D-9131-4245-A7BE-1A7384D5ADA0}" name="100m Lifesaver2"/>
     <tableColumn id="12" xr3:uid="{D9D6CF56-869C-4DDE-9886-572D4E523A8F}" name="200m Superlifesaver2"/>
@@ -8833,133 +8833,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:78" s="39" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="127">
+      <c r="A1" s="108">
         <v>2025</v>
       </c>
       <c r="B1" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="C1" s="108" t="s">
+      <c r="C1" s="109" t="s">
         <v>207</v>
       </c>
-      <c r="D1" s="108"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="112" t="s">
+      <c r="D1" s="109"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="111" t="s">
         <v>208</v>
       </c>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="114"/>
-      <c r="K1" s="118" t="s">
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="114" t="s">
         <v>212</v>
       </c>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="120"/>
-      <c r="O1" s="110" t="s">
+      <c r="L1" s="115"/>
+      <c r="M1" s="115"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="134" t="s">
         <v>209</v>
       </c>
-      <c r="P1" s="110"/>
-      <c r="Q1" s="111"/>
-      <c r="R1" s="124" t="s">
+      <c r="P1" s="134"/>
+      <c r="Q1" s="135"/>
+      <c r="R1" s="136" t="s">
         <v>210</v>
       </c>
-      <c r="S1" s="125"/>
-      <c r="T1" s="125"/>
-      <c r="U1" s="125"/>
-      <c r="V1" s="126"/>
-      <c r="W1" s="121" t="s">
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="137"/>
+      <c r="V1" s="138"/>
+      <c r="W1" s="139" t="s">
         <v>213</v>
       </c>
-      <c r="X1" s="122"/>
-      <c r="Y1" s="122"/>
-      <c r="Z1" s="123"/>
+      <c r="X1" s="140"/>
+      <c r="Y1" s="140"/>
+      <c r="Z1" s="141"/>
       <c r="AA1"/>
       <c r="AB1" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="AC1" s="128" t="s">
+      <c r="AC1" s="117" t="s">
         <v>214</v>
       </c>
-      <c r="AD1" s="128"/>
-      <c r="AE1" s="129"/>
-      <c r="AF1" s="130" t="s">
+      <c r="AD1" s="117"/>
+      <c r="AE1" s="118"/>
+      <c r="AF1" s="119" t="s">
         <v>215</v>
       </c>
-      <c r="AG1" s="131"/>
-      <c r="AH1" s="131"/>
-      <c r="AI1" s="131"/>
-      <c r="AJ1" s="132"/>
-      <c r="AK1" s="133" t="s">
+      <c r="AG1" s="120"/>
+      <c r="AH1" s="120"/>
+      <c r="AI1" s="120"/>
+      <c r="AJ1" s="121"/>
+      <c r="AK1" s="122" t="s">
         <v>216</v>
       </c>
-      <c r="AL1" s="134"/>
-      <c r="AM1" s="134"/>
-      <c r="AN1" s="135"/>
-      <c r="AO1" s="136" t="s">
+      <c r="AL1" s="123"/>
+      <c r="AM1" s="123"/>
+      <c r="AN1" s="124"/>
+      <c r="AO1" s="125" t="s">
         <v>217</v>
       </c>
-      <c r="AP1" s="137"/>
-      <c r="AQ1" s="138"/>
-      <c r="AR1" s="139" t="s">
+      <c r="AP1" s="126"/>
+      <c r="AQ1" s="127"/>
+      <c r="AR1" s="128" t="s">
         <v>218</v>
       </c>
-      <c r="AS1" s="140"/>
-      <c r="AT1" s="140"/>
-      <c r="AU1" s="140"/>
-      <c r="AV1" s="141"/>
-      <c r="AW1" s="115" t="s">
+      <c r="AS1" s="129"/>
+      <c r="AT1" s="129"/>
+      <c r="AU1" s="129"/>
+      <c r="AV1" s="130"/>
+      <c r="AW1" s="131" t="s">
         <v>219</v>
       </c>
-      <c r="AX1" s="116"/>
-      <c r="AY1" s="116"/>
-      <c r="AZ1" s="117"/>
+      <c r="AX1" s="132"/>
+      <c r="AY1" s="132"/>
+      <c r="AZ1" s="133"/>
       <c r="BB1" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())-1," für: ", YEAR(TODAY()))</f>
         <v>in: 2025 für: 2026</v>
       </c>
-      <c r="BC1" s="108" t="s">
+      <c r="BC1" s="109" t="s">
         <v>220</v>
       </c>
-      <c r="BD1" s="108"/>
-      <c r="BE1" s="109"/>
-      <c r="BF1" s="112" t="s">
+      <c r="BD1" s="109"/>
+      <c r="BE1" s="110"/>
+      <c r="BF1" s="111" t="s">
         <v>221</v>
       </c>
-      <c r="BG1" s="113"/>
-      <c r="BH1" s="113"/>
-      <c r="BI1" s="113"/>
-      <c r="BJ1" s="114"/>
-      <c r="BK1" s="118" t="s">
+      <c r="BG1" s="112"/>
+      <c r="BH1" s="112"/>
+      <c r="BI1" s="112"/>
+      <c r="BJ1" s="113"/>
+      <c r="BK1" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="BL1" s="119"/>
-      <c r="BM1" s="119"/>
-      <c r="BN1" s="120"/>
-      <c r="BO1" s="110" t="s">
+      <c r="BL1" s="115"/>
+      <c r="BM1" s="115"/>
+      <c r="BN1" s="116"/>
+      <c r="BO1" s="134" t="s">
         <v>227</v>
       </c>
-      <c r="BP1" s="110"/>
-      <c r="BQ1" s="111"/>
-      <c r="BR1" s="124" t="s">
+      <c r="BP1" s="134"/>
+      <c r="BQ1" s="135"/>
+      <c r="BR1" s="136" t="s">
         <v>228</v>
       </c>
-      <c r="BS1" s="125"/>
-      <c r="BT1" s="125"/>
-      <c r="BU1" s="125"/>
-      <c r="BV1" s="126"/>
-      <c r="BW1" s="121" t="s">
+      <c r="BS1" s="137"/>
+      <c r="BT1" s="137"/>
+      <c r="BU1" s="137"/>
+      <c r="BV1" s="138"/>
+      <c r="BW1" s="139" t="s">
         <v>223</v>
       </c>
-      <c r="BX1" s="122"/>
-      <c r="BY1" s="122"/>
-      <c r="BZ1" s="123"/>
+      <c r="BX1" s="140"/>
+      <c r="BY1" s="140"/>
+      <c r="BZ1" s="141"/>
     </row>
     <row r="2" spans="1:78" s="93" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="127"/>
+      <c r="A2" s="108"/>
       <c r="B2" s="45" t="s">
         <v>211</v>
       </c>
@@ -9260,7 +9260,7 @@
       </c>
     </row>
     <row r="3" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="127"/>
+      <c r="A3" s="108"/>
       <c r="B3" s="46" t="s">
         <v>0</v>
       </c>
@@ -9513,7 +9513,7 @@
       </c>
     </row>
     <row r="4" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A4" s="127"/>
+      <c r="A4" s="108"/>
       <c r="B4" s="46" t="s">
         <v>179</v>
       </c>
@@ -9765,7 +9765,7 @@
       </c>
     </row>
     <row r="5" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A5" s="127"/>
+      <c r="A5" s="108"/>
       <c r="B5" s="46" t="s">
         <v>180</v>
       </c>
@@ -10017,7 +10017,7 @@
       </c>
     </row>
     <row r="6" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A6" s="127"/>
+      <c r="A6" s="108"/>
       <c r="B6" s="46" t="s">
         <v>181</v>
       </c>
@@ -10269,7 +10269,7 @@
       </c>
     </row>
     <row r="7" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A7" s="127"/>
+      <c r="A7" s="108"/>
       <c r="B7" s="46" t="s">
         <v>182</v>
       </c>
@@ -10521,7 +10521,7 @@
       </c>
     </row>
     <row r="8" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="127"/>
+      <c r="A8" s="108"/>
       <c r="B8" s="49" t="s">
         <v>4</v>
       </c>
@@ -10774,132 +10774,132 @@
     </row>
     <row r="9" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="10" spans="1:78" ht="18" x14ac:dyDescent="0.45">
-      <c r="A10" s="127">
+      <c r="A10" s="108">
         <v>2026</v>
       </c>
       <c r="B10" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="C10" s="108" t="s">
+      <c r="C10" s="109" t="s">
         <v>207</v>
       </c>
-      <c r="D10" s="108"/>
-      <c r="E10" s="109"/>
-      <c r="F10" s="112" t="s">
+      <c r="D10" s="109"/>
+      <c r="E10" s="110"/>
+      <c r="F10" s="111" t="s">
         <v>208</v>
       </c>
-      <c r="G10" s="113"/>
-      <c r="H10" s="113"/>
-      <c r="I10" s="113"/>
-      <c r="J10" s="114"/>
-      <c r="K10" s="118" t="s">
+      <c r="G10" s="112"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+      <c r="J10" s="113"/>
+      <c r="K10" s="114" t="s">
         <v>212</v>
       </c>
-      <c r="L10" s="119"/>
-      <c r="M10" s="119"/>
-      <c r="N10" s="120"/>
-      <c r="O10" s="110" t="s">
+      <c r="L10" s="115"/>
+      <c r="M10" s="115"/>
+      <c r="N10" s="116"/>
+      <c r="O10" s="134" t="s">
         <v>209</v>
       </c>
-      <c r="P10" s="110"/>
-      <c r="Q10" s="111"/>
-      <c r="R10" s="124" t="s">
+      <c r="P10" s="134"/>
+      <c r="Q10" s="135"/>
+      <c r="R10" s="136" t="s">
         <v>210</v>
       </c>
-      <c r="S10" s="125"/>
-      <c r="T10" s="125"/>
-      <c r="U10" s="125"/>
-      <c r="V10" s="126"/>
-      <c r="W10" s="121" t="s">
+      <c r="S10" s="137"/>
+      <c r="T10" s="137"/>
+      <c r="U10" s="137"/>
+      <c r="V10" s="138"/>
+      <c r="W10" s="139" t="s">
         <v>213</v>
       </c>
-      <c r="X10" s="122"/>
-      <c r="Y10" s="122"/>
-      <c r="Z10" s="123"/>
+      <c r="X10" s="140"/>
+      <c r="Y10" s="140"/>
+      <c r="Z10" s="141"/>
       <c r="AB10" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="AC10" s="128" t="s">
+      <c r="AC10" s="117" t="s">
         <v>214</v>
       </c>
-      <c r="AD10" s="128"/>
-      <c r="AE10" s="129"/>
-      <c r="AF10" s="130" t="s">
+      <c r="AD10" s="117"/>
+      <c r="AE10" s="118"/>
+      <c r="AF10" s="119" t="s">
         <v>215</v>
       </c>
-      <c r="AG10" s="131"/>
-      <c r="AH10" s="131"/>
-      <c r="AI10" s="131"/>
-      <c r="AJ10" s="132"/>
-      <c r="AK10" s="133" t="s">
+      <c r="AG10" s="120"/>
+      <c r="AH10" s="120"/>
+      <c r="AI10" s="120"/>
+      <c r="AJ10" s="121"/>
+      <c r="AK10" s="122" t="s">
         <v>216</v>
       </c>
-      <c r="AL10" s="134"/>
-      <c r="AM10" s="134"/>
-      <c r="AN10" s="135"/>
-      <c r="AO10" s="136" t="s">
+      <c r="AL10" s="123"/>
+      <c r="AM10" s="123"/>
+      <c r="AN10" s="124"/>
+      <c r="AO10" s="125" t="s">
         <v>217</v>
       </c>
-      <c r="AP10" s="137"/>
-      <c r="AQ10" s="138"/>
-      <c r="AR10" s="139" t="s">
+      <c r="AP10" s="126"/>
+      <c r="AQ10" s="127"/>
+      <c r="AR10" s="128" t="s">
         <v>218</v>
       </c>
-      <c r="AS10" s="140"/>
-      <c r="AT10" s="140"/>
-      <c r="AU10" s="140"/>
-      <c r="AV10" s="141"/>
-      <c r="AW10" s="115" t="s">
+      <c r="AS10" s="129"/>
+      <c r="AT10" s="129"/>
+      <c r="AU10" s="129"/>
+      <c r="AV10" s="130"/>
+      <c r="AW10" s="131" t="s">
         <v>219</v>
       </c>
-      <c r="AX10" s="116"/>
-      <c r="AY10" s="116"/>
-      <c r="AZ10" s="117"/>
+      <c r="AX10" s="132"/>
+      <c r="AY10" s="132"/>
+      <c r="AZ10" s="133"/>
       <c r="BB10" s="44" t="str">
         <f ca="1">CONCATENATE("in: ",YEAR(TODAY())," für: ", YEAR(TODAY())+1)</f>
         <v>in: 2026 für: 2027</v>
       </c>
-      <c r="BC10" s="108" t="s">
+      <c r="BC10" s="109" t="s">
         <v>220</v>
       </c>
-      <c r="BD10" s="108"/>
-      <c r="BE10" s="109"/>
-      <c r="BF10" s="112" t="s">
+      <c r="BD10" s="109"/>
+      <c r="BE10" s="110"/>
+      <c r="BF10" s="111" t="s">
         <v>221</v>
       </c>
-      <c r="BG10" s="113"/>
-      <c r="BH10" s="113"/>
-      <c r="BI10" s="113"/>
-      <c r="BJ10" s="114"/>
-      <c r="BK10" s="118" t="s">
+      <c r="BG10" s="112"/>
+      <c r="BH10" s="112"/>
+      <c r="BI10" s="112"/>
+      <c r="BJ10" s="113"/>
+      <c r="BK10" s="114" t="s">
         <v>222</v>
       </c>
-      <c r="BL10" s="119"/>
-      <c r="BM10" s="119"/>
-      <c r="BN10" s="120"/>
-      <c r="BO10" s="110" t="s">
+      <c r="BL10" s="115"/>
+      <c r="BM10" s="115"/>
+      <c r="BN10" s="116"/>
+      <c r="BO10" s="134" t="s">
         <v>227</v>
       </c>
-      <c r="BP10" s="110"/>
-      <c r="BQ10" s="111"/>
-      <c r="BR10" s="124" t="s">
+      <c r="BP10" s="134"/>
+      <c r="BQ10" s="135"/>
+      <c r="BR10" s="136" t="s">
         <v>228</v>
       </c>
-      <c r="BS10" s="125"/>
-      <c r="BT10" s="125"/>
-      <c r="BU10" s="125"/>
-      <c r="BV10" s="126"/>
-      <c r="BW10" s="121" t="s">
+      <c r="BS10" s="137"/>
+      <c r="BT10" s="137"/>
+      <c r="BU10" s="137"/>
+      <c r="BV10" s="138"/>
+      <c r="BW10" s="139" t="s">
         <v>223</v>
       </c>
-      <c r="BX10" s="122"/>
-      <c r="BY10" s="122"/>
-      <c r="BZ10" s="123"/>
+      <c r="BX10" s="140"/>
+      <c r="BY10" s="140"/>
+      <c r="BZ10" s="141"/>
     </row>
     <row r="11" spans="1:78" ht="21.4" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="127"/>
+      <c r="A11" s="108"/>
       <c r="B11" s="45" t="s">
         <v>211</v>
       </c>
@@ -11200,7 +11200,7 @@
       </c>
     </row>
     <row r="12" spans="1:78" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="127"/>
+      <c r="A12" s="108"/>
       <c r="B12" s="46" t="s">
         <v>0</v>
       </c>
@@ -11452,7 +11452,7 @@
       </c>
     </row>
     <row r="13" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A13" s="127"/>
+      <c r="A13" s="108"/>
       <c r="B13" s="46" t="s">
         <v>179</v>
       </c>
@@ -11704,7 +11704,7 @@
       </c>
     </row>
     <row r="14" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A14" s="127"/>
+      <c r="A14" s="108"/>
       <c r="B14" s="46" t="s">
         <v>180</v>
       </c>
@@ -11956,7 +11956,7 @@
       </c>
     </row>
     <row r="15" spans="1:78" x14ac:dyDescent="0.45">
-      <c r="A15" s="127"/>
+      <c r="A15" s="108"/>
       <c r="B15" s="46" t="s">
         <v>181</v>
       </c>
@@ -12208,7 +12208,7 @@
       </c>
     </row>
     <row r="16" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="127"/>
+      <c r="A16" s="108"/>
       <c r="B16" s="46" t="s">
         <v>182</v>
       </c>
@@ -12460,7 +12460,7 @@
       </c>
     </row>
     <row r="17" spans="1:78" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="127"/>
+      <c r="A17" s="108"/>
       <c r="B17" s="49" t="s">
         <v>4</v>
       </c>
@@ -12927,6 +12927,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="AW10:AZ10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="W10:Z10"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="R10:V10"/>
+    <mergeCell ref="BO10:BQ10"/>
+    <mergeCell ref="BR10:BV10"/>
+    <mergeCell ref="BW10:BZ10"/>
+    <mergeCell ref="BC1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BO1:BQ1"/>
+    <mergeCell ref="BR1:BV1"/>
+    <mergeCell ref="BW1:BZ1"/>
     <mergeCell ref="A1:A8"/>
     <mergeCell ref="A10:A17"/>
     <mergeCell ref="BC10:BE10"/>
@@ -12943,28 +12965,6 @@
     <mergeCell ref="AK10:AN10"/>
     <mergeCell ref="AO10:AQ10"/>
     <mergeCell ref="AR10:AV10"/>
-    <mergeCell ref="BO10:BQ10"/>
-    <mergeCell ref="BR10:BV10"/>
-    <mergeCell ref="BW10:BZ10"/>
-    <mergeCell ref="BC1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BK1:BN1"/>
-    <mergeCell ref="BO1:BQ1"/>
-    <mergeCell ref="BR1:BV1"/>
-    <mergeCell ref="BW1:BZ1"/>
-    <mergeCell ref="AW10:AZ10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="W10:Z10"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="R1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="R10:V10"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F10:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="AC3:AZ8">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
@@ -17370,19 +17370,19 @@
         <v>125</v>
       </c>
       <c r="C2" s="24">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" s="24">
         <v>18</v>
       </c>
       <c r="E2" s="26">
-        <v>45839</v>
+        <v>45835</v>
       </c>
       <c r="F2" s="26">
-        <v>46193</v>
+        <v>46562</v>
       </c>
       <c r="G2" s="26">
-        <v>46023</v>
+        <v>46388</v>
       </c>
       <c r="H2" s="24" t="s">
         <v>139</v>
@@ -17396,40 +17396,40 @@
         <v>10</v>
       </c>
       <c r="M2" s="27">
-        <v>4.6817129629629634E-4</v>
+        <v>4.6226851851851849E-4</v>
       </c>
       <c r="N2" s="27">
-        <v>7.4872685185185188E-4</v>
+        <v>7.3530092592592592E-4</v>
       </c>
       <c r="O2" s="27">
-        <v>9.9224537037037033E-4</v>
+        <v>9.7326388888888896E-4</v>
       </c>
       <c r="P2" s="27">
-        <v>7.8888888888888889E-4</v>
+        <v>7.7465277777777786E-4</v>
       </c>
       <c r="Q2" s="27">
-        <v>1.9605324074074074E-3</v>
+        <v>1.8885416666666668E-3</v>
       </c>
       <c r="R2" s="27">
-        <v>1.7837962962962963E-3</v>
+        <v>1.7290509259259258E-3</v>
       </c>
       <c r="S2" s="27">
-        <v>4.803240740740741E-4</v>
+        <v>4.7627314814814814E-4</v>
       </c>
       <c r="T2" s="27">
-        <v>7.8599537037037039E-4</v>
+        <v>7.5960648148148144E-4</v>
       </c>
       <c r="U2" s="27">
-        <v>1.0240740740740742E-3</v>
+        <v>9.9270833333333329E-4</v>
       </c>
       <c r="V2" s="27">
-        <v>8.2766203703703712E-4</v>
+        <v>8.0370370370370372E-4</v>
       </c>
       <c r="W2" s="27">
-        <v>2.0114583333333334E-3</v>
+        <v>1.9607638888888891E-3</v>
       </c>
       <c r="X2" s="27">
-        <v>1.8332175925925925E-3</v>
+        <v>1.8109953703703704E-3</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.45">
@@ -17440,19 +17440,19 @@
         <v>143</v>
       </c>
       <c r="C3" s="24">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" s="24">
         <v>18</v>
       </c>
       <c r="E3" s="26">
-        <v>45839</v>
+        <v>45835</v>
       </c>
       <c r="F3" s="26">
-        <v>46193</v>
+        <v>46562</v>
       </c>
       <c r="G3" s="26">
-        <v>46023</v>
+        <v>46388</v>
       </c>
       <c r="H3" s="24" t="s">
         <v>139</v>
@@ -17466,40 +17466,40 @@
         <v>10</v>
       </c>
       <c r="M3" s="27">
-        <v>3.9178240740740742E-4</v>
+        <v>3.8715277777777782E-4</v>
       </c>
       <c r="N3" s="27">
-        <v>6.310185185185186E-4</v>
+        <v>5.9745370370370367E-4</v>
       </c>
       <c r="O3" s="27">
-        <v>8.5555555555555558E-4</v>
+        <v>8.3553240740740734E-4</v>
       </c>
       <c r="P3" s="27">
-        <v>7.0196759259259257E-4</v>
+        <v>6.75462962962963E-4</v>
       </c>
       <c r="Q3" s="27">
-        <v>1.7359953703703704E-3</v>
+        <v>1.7269675925925927E-3</v>
       </c>
       <c r="R3" s="27">
-        <v>1.6295138888888889E-3</v>
+        <v>1.603935185185185E-3</v>
       </c>
       <c r="S3" s="27">
-        <v>4.1747685185185187E-4</v>
+        <v>3.9942129629629626E-4</v>
       </c>
       <c r="T3" s="27">
-        <v>6.7627314814814818E-4</v>
+        <v>6.3472222222222228E-4</v>
       </c>
       <c r="U3" s="27">
-        <v>8.9861111111111109E-4</v>
+        <v>8.5949074074074085E-4</v>
       </c>
       <c r="V3" s="27">
-        <v>7.2384259259259255E-4</v>
+        <v>7.0856481481481476E-4</v>
       </c>
       <c r="W3" s="27">
-        <v>1.8050925925925927E-3</v>
+        <v>1.7791666666666667E-3</v>
       </c>
       <c r="X3" s="27">
-        <v>1.7003472222222222E-3</v>
+        <v>1.6371527777777777E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>